<commit_message>
Lanzar Beta-1.0.6 con personalizacion de color y ajustes de desafios.
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/resources/desafios.xlsx
+++ b/public/resources/desafios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F69F7584-4FFD-49B8-99B7-9A37826F3AF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04B03140-37C9-4EA0-AF2E-4E17A269114C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="36">
   <si>
     <t>nombre</t>
   </si>
@@ -90,12 +90,6 @@
     <t>Killer Croc</t>
   </si>
   <si>
-    <t>Sinestro</t>
-  </si>
-  <si>
-    <t>Parallax</t>
-  </si>
-  <si>
     <t>Bane</t>
   </si>
   <si>
@@ -129,28 +123,16 @@
     <t>Derrota a los villanos fugados de Black Gate</t>
   </si>
   <si>
-    <t>Sinestro Corps: Primer Contacto</t>
-  </si>
-  <si>
-    <t>Enfréntate a los linternas amarillas.</t>
-  </si>
-  <si>
-    <t>Feena Sik</t>
-  </si>
-  <si>
-    <t>Lyssa Drak</t>
-  </si>
-  <si>
-    <t>Derrotar al Miedo</t>
-  </si>
-  <si>
-    <t>Derrota a Sinestro.</t>
-  </si>
-  <si>
-    <t>Sinestro Corps: Invasión</t>
-  </si>
-  <si>
-    <t>Derrota a todos los miembros de Sinestro Corps</t>
+    <t>cartas</t>
+  </si>
+  <si>
+    <t>faccion</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>V</t>
   </si>
 </sst>
 </file>
@@ -172,7 +154,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -217,7 +199,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor rgb="FFFFCCCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF9999"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF6969"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -249,7 +243,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -286,6 +280,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -295,6 +307,11 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFF6969"/>
+      <color rgb="FFFF5050"/>
+      <color rgb="FFFF7C80"/>
+      <color rgb="FFFF9999"/>
+      <color rgb="FFFFCCCC"/>
       <color rgb="FF6DD17E"/>
       <color rgb="FF50C864"/>
       <color rgb="FFCC66FF"/>
@@ -574,338 +591,404 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="43.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="57.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="43.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="57.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" s="2">
+        <v>25</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="2">
         <v>1</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="F2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="G2" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="H2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
-      <c r="L2" s="2">
-        <v>0</v>
-      </c>
+      <c r="L2" s="2"/>
       <c r="M2" s="2">
         <v>0</v>
       </c>
       <c r="N2" s="2">
+        <v>0</v>
+      </c>
+      <c r="O2" s="2">
         <v>50</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P2" s="5"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="4">
+        <v>26</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="4">
         <v>1</v>
       </c>
-      <c r="E3" s="8"/>
       <c r="F3" s="8"/>
       <c r="G3" s="8"/>
-      <c r="H3" s="4"/>
+      <c r="H3" s="8"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
-      <c r="K3" s="8" t="s">
+      <c r="K3" s="4"/>
+      <c r="L3" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="4">
-        <v>0</v>
-      </c>
       <c r="M3" s="4">
         <v>0</v>
       </c>
       <c r="N3" s="4">
+        <v>0</v>
+      </c>
+      <c r="O3" s="4">
         <v>100</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P3" s="8"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D4" s="3">
+        <v>28</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="3">
         <v>1</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="H4" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="I4" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="9" t="s">
-        <v>25</v>
-      </c>
       <c r="J4" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3">
-        <v>0</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="K4" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="11"/>
       <c r="M4" s="3">
         <v>0</v>
       </c>
       <c r="N4" s="3">
+        <v>0</v>
+      </c>
+      <c r="O4" s="3">
         <v>150</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P4" s="8"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="10">
         <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" s="10">
+        <v>30</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="10">
         <v>1</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="F5" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="G5" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="H5" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="11"/>
       <c r="I5" s="11"/>
       <c r="J5" s="11"/>
-      <c r="K5" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="L5" s="10">
+      <c r="K5" s="11"/>
+      <c r="L5" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="M5" s="10">
         <v>1</v>
       </c>
-      <c r="M5" s="10">
-        <v>0</v>
-      </c>
       <c r="N5" s="10">
+        <v>0</v>
+      </c>
+      <c r="O5" s="10">
         <v>200</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P5" s="8"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="12">
-        <v>2</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="H6" s="12"/>
+        <v>25</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="12">
+        <v>1</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>15</v>
+      </c>
       <c r="I6" s="12"/>
       <c r="J6" s="12"/>
       <c r="K6" s="12"/>
-      <c r="L6" s="12">
-        <v>0</v>
-      </c>
+      <c r="L6" s="12"/>
       <c r="M6" s="12">
         <v>0</v>
       </c>
       <c r="N6" s="12">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="5">
-        <v>5</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="5">
+        <v>0</v>
+      </c>
+      <c r="O6" s="12">
+        <v>50</v>
+      </c>
+      <c r="P6" s="5"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="14">
+        <v>1</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="14">
+        <v>1</v>
+      </c>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="M7" s="14">
+        <v>0</v>
+      </c>
+      <c r="N7" s="14">
+        <v>0</v>
+      </c>
+      <c r="O7" s="14">
+        <v>100</v>
+      </c>
+      <c r="P7" s="8"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="16">
         <v>2</v>
       </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="6" t="s">
+      <c r="B8" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="16">
+        <v>1</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L8" s="6"/>
+      <c r="M8" s="16">
+        <v>0</v>
+      </c>
+      <c r="N8" s="16">
+        <v>0</v>
+      </c>
+      <c r="O8" s="16">
+        <v>150</v>
+      </c>
+      <c r="P8" s="8"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="17">
+        <v>3</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="17">
+        <v>1</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="I9" s="18"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="18"/>
+      <c r="L9" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="L7" s="5">
+      <c r="M9" s="17">
         <v>1</v>
       </c>
-      <c r="M7" s="5">
-        <v>1</v>
-      </c>
-      <c r="N7" s="5">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="5">
-        <v>6</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" s="5">
-        <v>2</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="L8" s="5">
-        <v>1</v>
-      </c>
-      <c r="M8" s="5">
-        <v>1</v>
-      </c>
-      <c r="N8" s="5">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N9" s="17">
+        <v>0</v>
+      </c>
+      <c r="O9" s="17">
+        <v>200</v>
+      </c>
+      <c r="P9" s="8"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -920,8 +1003,9 @@
       <c r="L10" s="5"/>
       <c r="M10" s="5"/>
       <c r="N10" s="5"/>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O10" s="5"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -936,8 +1020,9 @@
       <c r="L11" s="5"/>
       <c r="M11" s="5"/>
       <c r="N11" s="5"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O11" s="5"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -952,8 +1037,9 @@
       <c r="L12" s="5"/>
       <c r="M12" s="5"/>
       <c r="N12" s="5"/>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O12" s="5"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -968,8 +1054,9 @@
       <c r="L13" s="5"/>
       <c r="M13" s="5"/>
       <c r="N13" s="5"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O13" s="5"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -984,8 +1071,9 @@
       <c r="L14" s="5"/>
       <c r="M14" s="5"/>
       <c r="N14" s="5"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O14" s="5"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1000,8 +1088,9 @@
       <c r="L15" s="5"/>
       <c r="M15" s="5"/>
       <c r="N15" s="5"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O15" s="5"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -1016,8 +1105,9 @@
       <c r="L16" s="5"/>
       <c r="M16" s="5"/>
       <c r="N16" s="5"/>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O16" s="5"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1032,8 +1122,9 @@
       <c r="L17" s="5"/>
       <c r="M17" s="5"/>
       <c r="N17" s="5"/>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O17" s="5"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -1048,8 +1139,9 @@
       <c r="L18" s="5"/>
       <c r="M18" s="5"/>
       <c r="N18" s="5"/>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O18" s="5"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -1064,8 +1156,9 @@
       <c r="L19" s="5"/>
       <c r="M19" s="5"/>
       <c r="N19" s="5"/>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O19" s="5"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -1080,8 +1173,9 @@
       <c r="L20" s="5"/>
       <c r="M20" s="5"/>
       <c r="N20" s="5"/>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O20" s="5"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -1096,8 +1190,9 @@
       <c r="L21" s="5"/>
       <c r="M21" s="5"/>
       <c r="N21" s="5"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O21" s="5"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -1112,6 +1207,7 @@
       <c r="L22" s="5"/>
       <c r="M22" s="5"/>
       <c r="N22" s="5"/>
+      <c r="O22" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
Corrige /update-user tras guardado y flujo de apertura de sobres
- server: define docRefUsuario antes de getDoc en POST /update-user (evitaba 500 tras guardado correcto).

- coleccion: errores con status/codigo y reintentos ante 409 al persistir apertura de sobre.

- Actualiza desafios (HTML/JS), cartas.xlsx y desafios.xlsx.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/desafios.xlsx
+++ b/public/resources/desafios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D24237FD-8E3C-4216-9A44-9868759FBBCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2056CC57-C7A4-41FD-AD46-A059359AA68B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="309">
   <si>
     <t>nombre</t>
   </si>
@@ -517,6 +517,441 @@
   </si>
   <si>
     <t>King Shark</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>La Última Defensa de la Tierra</t>
+  </si>
+  <si>
+    <t>Derrota a la Liga de la Justicia y hazte con el control del planeta Tierra.</t>
+  </si>
+  <si>
+    <t>Batman</t>
+  </si>
+  <si>
+    <t>Wonder Woman</t>
+  </si>
+  <si>
+    <t>Flash</t>
+  </si>
+  <si>
+    <t>Aquaman</t>
+  </si>
+  <si>
+    <t>Hal Jordan</t>
+  </si>
+  <si>
+    <t>Martian Manhunter</t>
+  </si>
+  <si>
+    <t>Superman</t>
+  </si>
+  <si>
+    <t>Crisis sobre Metrópolis</t>
+  </si>
+  <si>
+    <t>Acaba con todos los Héroes de la Liga de la Justicia y siembra el caos en Metrópolis</t>
+  </si>
+  <si>
+    <t>Shazam</t>
+  </si>
+  <si>
+    <t>Cyborg</t>
+  </si>
+  <si>
+    <t>Hawkgirl</t>
+  </si>
+  <si>
+    <t>Hawkman</t>
+  </si>
+  <si>
+    <t>Sol Rojo</t>
+  </si>
+  <si>
+    <t>Enfréntate y derrota a todos los miembros de la Casa de EL</t>
+  </si>
+  <si>
+    <t>Krypto</t>
+  </si>
+  <si>
+    <t>Steel</t>
+  </si>
+  <si>
+    <t>Superboy</t>
+  </si>
+  <si>
+    <t>Supergirl</t>
+  </si>
+  <si>
+    <t>Power Girl</t>
+  </si>
+  <si>
+    <t>Las Profundidades de Atlantis</t>
+  </si>
+  <si>
+    <t>Derrota a los protectores de Atlantis.</t>
+  </si>
+  <si>
+    <t>Atlanna</t>
+  </si>
+  <si>
+    <t>Aqualad</t>
+  </si>
+  <si>
+    <t>Mera</t>
+  </si>
+  <si>
+    <t>Alas de Thanagar</t>
+  </si>
+  <si>
+    <t>Enfrentate a los Nuevos Dioses en una batalla desenfrenada.</t>
+  </si>
+  <si>
+    <t>Highfather</t>
+  </si>
+  <si>
+    <t>Mister Miracle</t>
+  </si>
+  <si>
+    <t>Big Barda</t>
+  </si>
+  <si>
+    <t>Bekka</t>
+  </si>
+  <si>
+    <t>Orion</t>
+  </si>
+  <si>
+    <t>Adam Strange</t>
+  </si>
+  <si>
+    <t>Protocolo Omega</t>
+  </si>
+  <si>
+    <t>Derrota a los héroes con la mejor y más peligrosa tecnología antes de se interpongan en tú camino.</t>
+  </si>
+  <si>
+    <t>Rocket</t>
+  </si>
+  <si>
+    <t>Static</t>
+  </si>
+  <si>
+    <t>Hardware</t>
+  </si>
+  <si>
+    <t>Mr. Terrific</t>
+  </si>
+  <si>
+    <t>Blue Beetle</t>
+  </si>
+  <si>
+    <t>Firestorm</t>
+  </si>
+  <si>
+    <t>Red Tornado</t>
+  </si>
+  <si>
+    <t>Captain Atom</t>
+  </si>
+  <si>
+    <t>Caos en Dakota</t>
+  </si>
+  <si>
+    <t>Derrota a los Héroes que protegen Dakota y siembra el caos en la ciudad.</t>
+  </si>
+  <si>
+    <t>Icon</t>
+  </si>
+  <si>
+    <t>El Corazón de la Tierra</t>
+  </si>
+  <si>
+    <t>Enfrentate a la Ira del Verde y derrota a todos los Héroes que protegen la vida en el planeta Tierra.</t>
+  </si>
+  <si>
+    <t>Swamp Thing</t>
+  </si>
+  <si>
+    <t>Doctor Light</t>
+  </si>
+  <si>
+    <t>Vixen</t>
+  </si>
+  <si>
+    <t>Beast Boy</t>
+  </si>
+  <si>
+    <t>Hielo</t>
+  </si>
+  <si>
+    <t>Fuego</t>
+  </si>
+  <si>
+    <t>Generación Heróica</t>
+  </si>
+  <si>
+    <t>La Amenaza Interior</t>
+  </si>
+  <si>
+    <t>Titanes Unidos</t>
+  </si>
+  <si>
+    <t>Enfrentate a la nueva generación de héroes que protege la tierra. Los Titanes.</t>
+  </si>
+  <si>
+    <t>Donna Troy</t>
+  </si>
+  <si>
+    <t>Raven</t>
+  </si>
+  <si>
+    <t>La Hija de Trigon</t>
+  </si>
+  <si>
+    <t>Sobrevive a la sombra que oculta el alma de Raven. Si puedes.</t>
+  </si>
+  <si>
+    <t>Enfrentate a todos los Titanes unidos antes de que desbaraten tus planes.</t>
+  </si>
+  <si>
+    <t>Wonder Girl</t>
+  </si>
+  <si>
+    <t>Kid Flash</t>
+  </si>
+  <si>
+    <t>Starfire</t>
+  </si>
+  <si>
+    <t>Una última batalla contra los Titanes más poderosos que decidirá el destino de todos.</t>
+  </si>
+  <si>
+    <t>Nightwing</t>
+  </si>
+  <si>
+    <t>La última linea temporal</t>
+  </si>
+  <si>
+    <t>Viaja al siglo XXXI y enfréntate a los Héroes más poderosos de la Legión de Superhéroes</t>
+  </si>
+  <si>
+    <t>Shadow Lass</t>
+  </si>
+  <si>
+    <t>Brainiac-5</t>
+  </si>
+  <si>
+    <t>Lightning Lad</t>
+  </si>
+  <si>
+    <t>Cosmic Boy</t>
+  </si>
+  <si>
+    <t>Saturn Girl</t>
+  </si>
+  <si>
+    <t>Hijas de Themyscira</t>
+  </si>
+  <si>
+    <t>Sobrevive a la furia de las Amazonas más poderosas de la Tierra.</t>
+  </si>
+  <si>
+    <t>Yara Flor</t>
+  </si>
+  <si>
+    <t>Artemis</t>
+  </si>
+  <si>
+    <t>Nubia</t>
+  </si>
+  <si>
+    <t>Trinity</t>
+  </si>
+  <si>
+    <t>Héroes del mañana</t>
+  </si>
+  <si>
+    <t>No permitas que la nueva generación de Héroes desbarate tus planes. Derrótalos a todos.</t>
+  </si>
+  <si>
+    <t>Jesse Quick</t>
+  </si>
+  <si>
+    <t>Galaxy</t>
+  </si>
+  <si>
+    <t>Dreamer</t>
+  </si>
+  <si>
+    <t>Faruka</t>
+  </si>
+  <si>
+    <t>La paradoja de Booster</t>
+  </si>
+  <si>
+    <t>Salta en el tiempo, afronta paradojas y bucles temporales, en una batalla frenética contra los Héroes más peculiares de todas las lineas temporales.</t>
+  </si>
+  <si>
+    <t>Ray Palmer</t>
+  </si>
+  <si>
+    <t>Atom</t>
+  </si>
+  <si>
+    <t>Plastic Man</t>
+  </si>
+  <si>
+    <t>Booster Gold</t>
+  </si>
+  <si>
+    <t>El Libro del destino</t>
+  </si>
+  <si>
+    <t>Maldiciones, dimensiones mágicas. Derrota a la magia más poderosa que poseen los héroes.</t>
+  </si>
+  <si>
+    <t>Amethyst</t>
+  </si>
+  <si>
+    <t>Etrigan</t>
+  </si>
+  <si>
+    <t>Madame Xanadu</t>
+  </si>
+  <si>
+    <t>Sombras de la casa del misterio</t>
+  </si>
+  <si>
+    <t>John Constantine y su séquito de bichos raros necesita una buena lección.</t>
+  </si>
+  <si>
+    <t>John Constantine</t>
+  </si>
+  <si>
+    <t>Zatanna</t>
+  </si>
+  <si>
+    <t>Pandora</t>
+  </si>
+  <si>
+    <t>Doctor Fate</t>
+  </si>
+  <si>
+    <t>El reino de los condenados</t>
+  </si>
+  <si>
+    <t>Deadman</t>
+  </si>
+  <si>
+    <t>Maleficio inquebrantable</t>
+  </si>
+  <si>
+    <t>Derrota a los héroes en una batalla donde la magia decidirá el destino de todos.</t>
+  </si>
+  <si>
+    <t>Enfrentate a la magia más poderosa y trata de salir con vida.</t>
+  </si>
+  <si>
+    <t>Sector 2814</t>
+  </si>
+  <si>
+    <t>El cuerpo de Linternas verdes está en la zona. Deshazte de ellos antes de que se vuelvan un problema.</t>
+  </si>
+  <si>
+    <t>Simon Baz</t>
+  </si>
+  <si>
+    <t>Arisia Rrab</t>
+  </si>
+  <si>
+    <t>Jo Mullein</t>
+  </si>
+  <si>
+    <t>Los caballeros esmeralda</t>
+  </si>
+  <si>
+    <t>Los cuerpos de linternas verdes han pedido refuerzos. No dejes que John Stewart te derrote</t>
+  </si>
+  <si>
+    <t>Kyle Rayner</t>
+  </si>
+  <si>
+    <t>Abin Sur</t>
+  </si>
+  <si>
+    <t>Jade</t>
+  </si>
+  <si>
+    <t>John Stewart</t>
+  </si>
+  <si>
+    <t>Guerra de los anillos</t>
+  </si>
+  <si>
+    <t>Derrota al cuerpo de linternas verdes al completo.</t>
+  </si>
+  <si>
+    <t>Guy Gardner</t>
+  </si>
+  <si>
+    <t>Jessica Cruz</t>
+  </si>
+  <si>
+    <t>La Caída de OA</t>
+  </si>
+  <si>
+    <t>La última resistencia de OA. Los linternas más poderosos, derrótalos y la victoria sobre la luz será tuya.</t>
+  </si>
+  <si>
+    <t>Sombras sobre Gotham</t>
+  </si>
+  <si>
+    <t>La Bat-Familia sigue azotando a las mafías y los malechores de Gotham. Acaba con ellos antes de que lo estropeen todo.</t>
+  </si>
+  <si>
+    <t>Huntress</t>
+  </si>
+  <si>
+    <t>Batwing</t>
+  </si>
+  <si>
+    <t>Signal</t>
+  </si>
+  <si>
+    <t>El Archivo Arkham</t>
+  </si>
+  <si>
+    <t>Ejecuta tu venganza sobre todos los justicieros que te encerraron en Arkham</t>
+  </si>
+  <si>
+    <t>Red Hood</t>
+  </si>
+  <si>
+    <t>Robin</t>
+  </si>
+  <si>
+    <t>Batgirl</t>
+  </si>
+  <si>
+    <t>La noche de los vigilantes</t>
+  </si>
+  <si>
+    <t>La Bat-Familia al completo ha salido de su madriguera. Es el momento de acabar con ellos de una vez por todas.</t>
+  </si>
+  <si>
+    <t>Batwoman</t>
+  </si>
+  <si>
+    <t>La venganza</t>
+  </si>
+  <si>
+    <t>Enfrentate al justiciero más temido de Gotham y a sus mejores discipulos.</t>
+  </si>
+  <si>
+    <t>Red Robin</t>
   </si>
 </sst>
 </file>
@@ -538,7 +973,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -581,6 +1016,30 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCCCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF9999"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF7C80"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF6969"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -609,7 +1068,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -644,7 +1103,33 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -653,12 +1138,12 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="FFCC99FF"/>
       <color rgb="FFFF6969"/>
-      <color rgb="FFFF5050"/>
       <color rgb="FFFF7C80"/>
       <color rgb="FFFF9999"/>
       <color rgb="FFFFCCCC"/>
+      <color rgb="FFCC99FF"/>
+      <color rgb="FFFF5050"/>
       <color rgb="FF6DD17E"/>
       <color rgb="FF50C864"/>
       <color rgb="FFCC66FF"/>
@@ -938,25 +1423,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P57"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="57.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.7109375" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" style="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.28515625" style="20" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.85546875" style="20" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="57.85546875" style="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" style="20" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="16.7109375" style="20" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" style="20" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.42578125" style="20" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.42578125" style="20" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19" style="20" customWidth="1"/>
+    <col min="12" max="12" width="18.85546875" style="20" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.28515625" style="20" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.5703125" style="20" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.140625" style="20"/>
+    <col min="16" max="16" width="17.7109375" style="20" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="20"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -1874,17 +2362,17 @@
         <v>110</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="10">
         <v>20</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="D22" s="12" t="s">
+      <c r="D22" s="10" t="s">
         <v>160</v>
       </c>
       <c r="E22" s="10">
@@ -1920,7 +2408,7 @@
       </c>
       <c r="P22" s="10"/>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="10">
         <v>21</v>
       </c>
@@ -1966,7 +2454,7 @@
       </c>
       <c r="P23" s="10"/>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="10">
         <v>22</v>
       </c>
@@ -2010,7 +2498,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="10">
         <v>23</v>
       </c>
@@ -2058,7 +2546,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="10">
         <v>24</v>
       </c>
@@ -2104,7 +2592,7 @@
       </c>
       <c r="P26" s="11"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="10">
         <v>25</v>
       </c>
@@ -2150,7 +2638,7 @@
       </c>
       <c r="P27" s="10"/>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="10">
         <v>26</v>
       </c>
@@ -2200,7 +2688,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="10">
         <v>27</v>
       </c>
@@ -2248,6 +2736,1254 @@
       </c>
       <c r="P29" s="11" t="s">
         <v>118</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="12">
+        <v>28</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="E30" s="12">
+        <v>1</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="G30" s="13" t="s">
+        <v>225</v>
+      </c>
+      <c r="H30" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="I30" s="12"/>
+      <c r="J30" s="12"/>
+      <c r="K30" s="12"/>
+      <c r="L30" s="12"/>
+      <c r="M30" s="12">
+        <v>0</v>
+      </c>
+      <c r="N30" s="12">
+        <v>0</v>
+      </c>
+      <c r="O30" s="12">
+        <v>50</v>
+      </c>
+      <c r="P30" s="12"/>
+    </row>
+    <row r="31" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="14">
+        <v>29</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>228</v>
+      </c>
+      <c r="E31" s="14">
+        <v>1</v>
+      </c>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
+      <c r="H31" s="15"/>
+      <c r="I31" s="14"/>
+      <c r="J31" s="14"/>
+      <c r="K31" s="14"/>
+      <c r="L31" s="15" t="s">
+        <v>226</v>
+      </c>
+      <c r="M31" s="14">
+        <v>0</v>
+      </c>
+      <c r="N31" s="14">
+        <v>0</v>
+      </c>
+      <c r="O31" s="14">
+        <v>100</v>
+      </c>
+      <c r="P31" s="15" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="16">
+        <v>30</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="D32" s="16" t="s">
+        <v>229</v>
+      </c>
+      <c r="E32" s="16">
+        <v>1</v>
+      </c>
+      <c r="F32" s="17" t="s">
+        <v>230</v>
+      </c>
+      <c r="G32" s="17" t="s">
+        <v>225</v>
+      </c>
+      <c r="H32" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="I32" s="17" t="s">
+        <v>226</v>
+      </c>
+      <c r="J32" s="17" t="s">
+        <v>232</v>
+      </c>
+      <c r="K32" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="L32" s="17"/>
+      <c r="M32" s="16">
+        <v>0</v>
+      </c>
+      <c r="N32" s="16">
+        <v>0</v>
+      </c>
+      <c r="O32" s="16">
+        <v>150</v>
+      </c>
+      <c r="P32" s="17"/>
+    </row>
+    <row r="33" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="18">
+        <v>31</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="C33" s="18" t="s">
+        <v>222</v>
+      </c>
+      <c r="D33" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="E33" s="18">
+        <v>1</v>
+      </c>
+      <c r="F33" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="G33" s="19" t="s">
+        <v>226</v>
+      </c>
+      <c r="H33" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="I33" s="19"/>
+      <c r="J33" s="19"/>
+      <c r="K33" s="19"/>
+      <c r="L33" s="19" t="s">
+        <v>232</v>
+      </c>
+      <c r="M33" s="18">
+        <v>1</v>
+      </c>
+      <c r="N33" s="18">
+        <v>0</v>
+      </c>
+      <c r="O33" s="18">
+        <v>200</v>
+      </c>
+      <c r="P33" s="19" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="12">
+        <v>32</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>293</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="E34" s="12">
+        <v>2</v>
+      </c>
+      <c r="F34" s="13" t="s">
+        <v>295</v>
+      </c>
+      <c r="G34" s="13" t="s">
+        <v>296</v>
+      </c>
+      <c r="H34" s="13" t="s">
+        <v>297</v>
+      </c>
+      <c r="I34" s="12"/>
+      <c r="J34" s="12"/>
+      <c r="K34" s="12"/>
+      <c r="L34" s="12"/>
+      <c r="M34" s="12"/>
+      <c r="N34" s="12"/>
+      <c r="O34" s="12">
+        <v>200</v>
+      </c>
+      <c r="P34" s="12"/>
+    </row>
+    <row r="35" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="14">
+        <v>33</v>
+      </c>
+      <c r="B35" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>298</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>299</v>
+      </c>
+      <c r="E35" s="14">
+        <v>2</v>
+      </c>
+      <c r="F35" s="15" t="s">
+        <v>300</v>
+      </c>
+      <c r="G35" s="15" t="s">
+        <v>234</v>
+      </c>
+      <c r="H35" s="15" t="s">
+        <v>301</v>
+      </c>
+      <c r="I35" s="14"/>
+      <c r="J35" s="14"/>
+      <c r="K35" s="14"/>
+      <c r="L35" s="15" t="s">
+        <v>302</v>
+      </c>
+      <c r="M35" s="14">
+        <v>0</v>
+      </c>
+      <c r="N35" s="14">
+        <v>0</v>
+      </c>
+      <c r="O35" s="14">
+        <v>250</v>
+      </c>
+      <c r="P35" s="15" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="16">
+        <v>34</v>
+      </c>
+      <c r="B36" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="D36" s="16" t="s">
+        <v>304</v>
+      </c>
+      <c r="E36" s="16">
+        <v>2</v>
+      </c>
+      <c r="F36" s="17" t="s">
+        <v>305</v>
+      </c>
+      <c r="G36" s="17" t="s">
+        <v>301</v>
+      </c>
+      <c r="H36" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="I36" s="17" t="s">
+        <v>302</v>
+      </c>
+      <c r="J36" s="17" t="s">
+        <v>300</v>
+      </c>
+      <c r="K36" s="17" t="s">
+        <v>167</v>
+      </c>
+      <c r="L36" s="17"/>
+      <c r="M36" s="16">
+        <v>0</v>
+      </c>
+      <c r="N36" s="16">
+        <v>0</v>
+      </c>
+      <c r="O36" s="16">
+        <v>300</v>
+      </c>
+      <c r="P36" s="17"/>
+    </row>
+    <row r="37" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="18">
+        <v>35</v>
+      </c>
+      <c r="B37" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="C37" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="D37" s="18" t="s">
+        <v>307</v>
+      </c>
+      <c r="E37" s="18">
+        <v>2</v>
+      </c>
+      <c r="F37" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="G37" s="19" t="s">
+        <v>302</v>
+      </c>
+      <c r="H37" s="19" t="s">
+        <v>308</v>
+      </c>
+      <c r="I37" s="19"/>
+      <c r="J37" s="19"/>
+      <c r="K37" s="19"/>
+      <c r="L37" s="19" t="s">
+        <v>167</v>
+      </c>
+      <c r="M37" s="18">
+        <v>1</v>
+      </c>
+      <c r="N37" s="18">
+        <v>0</v>
+      </c>
+      <c r="O37" s="18">
+        <v>350</v>
+      </c>
+      <c r="P37" s="19" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="12">
+        <v>36</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="E38" s="12">
+        <v>3</v>
+      </c>
+      <c r="F38" s="13" t="s">
+        <v>278</v>
+      </c>
+      <c r="G38" s="13" t="s">
+        <v>279</v>
+      </c>
+      <c r="H38" s="13" t="s">
+        <v>280</v>
+      </c>
+      <c r="I38" s="12"/>
+      <c r="J38" s="12"/>
+      <c r="K38" s="12"/>
+      <c r="L38" s="12"/>
+      <c r="M38" s="12">
+        <v>0</v>
+      </c>
+      <c r="N38" s="12">
+        <v>0</v>
+      </c>
+      <c r="O38" s="12">
+        <v>350</v>
+      </c>
+      <c r="P38" s="12"/>
+    </row>
+    <row r="39" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="14">
+        <v>37</v>
+      </c>
+      <c r="B39" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>281</v>
+      </c>
+      <c r="D39" s="14" t="s">
+        <v>282</v>
+      </c>
+      <c r="E39" s="14">
+        <v>3</v>
+      </c>
+      <c r="F39" s="15" t="s">
+        <v>283</v>
+      </c>
+      <c r="G39" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="H39" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="I39" s="14"/>
+      <c r="J39" s="14"/>
+      <c r="K39" s="14"/>
+      <c r="L39" s="15" t="s">
+        <v>286</v>
+      </c>
+      <c r="M39" s="14">
+        <v>0</v>
+      </c>
+      <c r="N39" s="14">
+        <v>0</v>
+      </c>
+      <c r="O39" s="14">
+        <v>400</v>
+      </c>
+      <c r="P39" s="15" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="16">
+        <v>38</v>
+      </c>
+      <c r="B40" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>287</v>
+      </c>
+      <c r="D40" s="16" t="s">
+        <v>288</v>
+      </c>
+      <c r="E40" s="16">
+        <v>3</v>
+      </c>
+      <c r="F40" s="17" t="s">
+        <v>289</v>
+      </c>
+      <c r="G40" s="17" t="s">
+        <v>283</v>
+      </c>
+      <c r="H40" s="17" t="s">
+        <v>278</v>
+      </c>
+      <c r="I40" s="17" t="s">
+        <v>290</v>
+      </c>
+      <c r="J40" s="17" t="s">
+        <v>286</v>
+      </c>
+      <c r="K40" s="17" t="s">
+        <v>171</v>
+      </c>
+      <c r="L40" s="17"/>
+      <c r="M40" s="16">
+        <v>0</v>
+      </c>
+      <c r="N40" s="16">
+        <v>0</v>
+      </c>
+      <c r="O40" s="16">
+        <v>450</v>
+      </c>
+      <c r="P40" s="17"/>
+    </row>
+    <row r="41" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="18">
+        <v>39</v>
+      </c>
+      <c r="B41" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="C41" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="D41" s="18" t="s">
+        <v>292</v>
+      </c>
+      <c r="E41" s="18">
+        <v>3</v>
+      </c>
+      <c r="F41" s="19" t="s">
+        <v>290</v>
+      </c>
+      <c r="G41" s="19" t="s">
+        <v>286</v>
+      </c>
+      <c r="H41" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="I41" s="19"/>
+      <c r="J41" s="19"/>
+      <c r="K41" s="19"/>
+      <c r="L41" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="M41" s="18">
+        <v>1</v>
+      </c>
+      <c r="N41" s="18">
+        <v>0</v>
+      </c>
+      <c r="O41" s="18">
+        <v>500</v>
+      </c>
+      <c r="P41" s="19" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="12">
+        <v>40</v>
+      </c>
+      <c r="B42" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="D42" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="E42" s="12">
+        <v>4</v>
+      </c>
+      <c r="F42" s="13" t="s">
+        <v>262</v>
+      </c>
+      <c r="G42" s="13" t="s">
+        <v>263</v>
+      </c>
+      <c r="H42" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="I42" s="12"/>
+      <c r="J42" s="12"/>
+      <c r="K42" s="12"/>
+      <c r="L42" s="12"/>
+      <c r="M42" s="12">
+        <v>0</v>
+      </c>
+      <c r="N42" s="12">
+        <v>0</v>
+      </c>
+      <c r="O42" s="12">
+        <v>500</v>
+      </c>
+      <c r="P42" s="12"/>
+    </row>
+    <row r="43" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="14">
+        <v>41</v>
+      </c>
+      <c r="B43" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="C43" s="14" t="s">
+        <v>265</v>
+      </c>
+      <c r="D43" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="E43" s="14">
+        <v>4</v>
+      </c>
+      <c r="F43" s="15" t="s">
+        <v>268</v>
+      </c>
+      <c r="G43" s="15" t="s">
+        <v>226</v>
+      </c>
+      <c r="H43" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="I43" s="14"/>
+      <c r="J43" s="14"/>
+      <c r="K43" s="14"/>
+      <c r="L43" s="15" t="s">
+        <v>267</v>
+      </c>
+      <c r="M43" s="14">
+        <v>0</v>
+      </c>
+      <c r="N43" s="14">
+        <v>0</v>
+      </c>
+      <c r="O43" s="14">
+        <v>550</v>
+      </c>
+      <c r="P43" s="15" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="16">
+        <v>42</v>
+      </c>
+      <c r="B44" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="C44" s="16" t="s">
+        <v>271</v>
+      </c>
+      <c r="D44" s="16" t="s">
+        <v>274</v>
+      </c>
+      <c r="E44" s="16">
+        <v>4</v>
+      </c>
+      <c r="F44" s="17" t="s">
+        <v>263</v>
+      </c>
+      <c r="G44" s="17" t="s">
+        <v>264</v>
+      </c>
+      <c r="H44" s="17" t="s">
+        <v>272</v>
+      </c>
+      <c r="I44" s="17" t="s">
+        <v>268</v>
+      </c>
+      <c r="J44" s="17" t="s">
+        <v>267</v>
+      </c>
+      <c r="K44" s="17" t="s">
+        <v>270</v>
+      </c>
+      <c r="L44" s="17"/>
+      <c r="M44" s="16">
+        <v>0</v>
+      </c>
+      <c r="N44" s="16">
+        <v>0</v>
+      </c>
+      <c r="O44" s="16">
+        <v>600</v>
+      </c>
+      <c r="P44" s="17"/>
+    </row>
+    <row r="45" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="18">
+        <v>43</v>
+      </c>
+      <c r="B45" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="C45" s="18" t="s">
+        <v>273</v>
+      </c>
+      <c r="D45" s="18" t="s">
+        <v>275</v>
+      </c>
+      <c r="E45" s="18">
+        <v>4</v>
+      </c>
+      <c r="F45" s="19" t="s">
+        <v>268</v>
+      </c>
+      <c r="G45" s="19" t="s">
+        <v>267</v>
+      </c>
+      <c r="H45" s="19" t="s">
+        <v>270</v>
+      </c>
+      <c r="I45" s="19"/>
+      <c r="J45" s="19"/>
+      <c r="K45" s="19"/>
+      <c r="L45" s="19" t="s">
+        <v>269</v>
+      </c>
+      <c r="M45" s="18">
+        <v>1</v>
+      </c>
+      <c r="N45" s="18">
+        <v>0</v>
+      </c>
+      <c r="O45" s="18">
+        <v>650</v>
+      </c>
+      <c r="P45" s="19" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="12">
+        <v>44</v>
+      </c>
+      <c r="B46" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>235</v>
+      </c>
+      <c r="D46" s="12" t="s">
+        <v>236</v>
+      </c>
+      <c r="E46" s="12">
+        <v>5</v>
+      </c>
+      <c r="F46" s="13" t="s">
+        <v>237</v>
+      </c>
+      <c r="G46" s="13" t="s">
+        <v>238</v>
+      </c>
+      <c r="H46" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="I46" s="12" t="s">
+        <v>240</v>
+      </c>
+      <c r="J46" s="12"/>
+      <c r="K46" s="12"/>
+      <c r="L46" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="M46" s="12">
+        <v>0</v>
+      </c>
+      <c r="N46" s="12">
+        <v>0</v>
+      </c>
+      <c r="O46" s="12">
+        <v>650</v>
+      </c>
+      <c r="P46" s="12" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="14">
+        <v>45</v>
+      </c>
+      <c r="B47" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="C47" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="D47" s="14" t="s">
+        <v>243</v>
+      </c>
+      <c r="E47" s="14">
+        <v>5</v>
+      </c>
+      <c r="F47" s="15" t="s">
+        <v>244</v>
+      </c>
+      <c r="G47" s="15" t="s">
+        <v>245</v>
+      </c>
+      <c r="H47" s="15" t="s">
+        <v>246</v>
+      </c>
+      <c r="I47" s="14" t="s">
+        <v>230</v>
+      </c>
+      <c r="J47" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="K47" s="14" t="s">
+        <v>247</v>
+      </c>
+      <c r="L47" s="15"/>
+      <c r="M47" s="14">
+        <v>0</v>
+      </c>
+      <c r="N47" s="14">
+        <v>0</v>
+      </c>
+      <c r="O47" s="14">
+        <v>700</v>
+      </c>
+      <c r="P47" s="15"/>
+    </row>
+    <row r="48" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="16">
+        <v>46</v>
+      </c>
+      <c r="B48" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="C48" s="16" t="s">
+        <v>248</v>
+      </c>
+      <c r="D48" s="16" t="s">
+        <v>249</v>
+      </c>
+      <c r="E48" s="16">
+        <v>5</v>
+      </c>
+      <c r="F48" s="17" t="s">
+        <v>253</v>
+      </c>
+      <c r="G48" s="17" t="s">
+        <v>206</v>
+      </c>
+      <c r="H48" s="17" t="s">
+        <v>250</v>
+      </c>
+      <c r="I48" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="J48" s="17" t="s">
+        <v>251</v>
+      </c>
+      <c r="K48" s="17" t="s">
+        <v>252</v>
+      </c>
+      <c r="L48" s="17"/>
+      <c r="M48" s="16">
+        <v>0</v>
+      </c>
+      <c r="N48" s="16">
+        <v>0</v>
+      </c>
+      <c r="O48" s="16">
+        <v>750</v>
+      </c>
+      <c r="P48" s="17"/>
+    </row>
+    <row r="49" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="18">
+        <v>47</v>
+      </c>
+      <c r="B49" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="C49" s="18" t="s">
+        <v>254</v>
+      </c>
+      <c r="D49" s="18" t="s">
+        <v>255</v>
+      </c>
+      <c r="E49" s="18">
+        <v>5</v>
+      </c>
+      <c r="F49" s="19" t="s">
+        <v>256</v>
+      </c>
+      <c r="G49" s="19" t="s">
+        <v>257</v>
+      </c>
+      <c r="H49" s="19" t="s">
+        <v>258</v>
+      </c>
+      <c r="I49" s="19"/>
+      <c r="J49" s="19"/>
+      <c r="K49" s="19"/>
+      <c r="L49" s="19" t="s">
+        <v>259</v>
+      </c>
+      <c r="M49" s="18">
+        <v>1</v>
+      </c>
+      <c r="N49" s="18">
+        <v>0</v>
+      </c>
+      <c r="O49" s="18">
+        <v>800</v>
+      </c>
+      <c r="P49" s="19" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="10">
+        <v>48</v>
+      </c>
+      <c r="B50" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="C50" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="D50" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="E50" s="10">
+        <v>6</v>
+      </c>
+      <c r="F50" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="G50" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="H50" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="I50" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="J50" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="K50" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="L50" s="10"/>
+      <c r="M50" s="10">
+        <v>1</v>
+      </c>
+      <c r="N50" s="10">
+        <v>1</v>
+      </c>
+      <c r="O50" s="10">
+        <v>800</v>
+      </c>
+      <c r="P50" s="10"/>
+    </row>
+    <row r="51" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="10">
+        <v>49</v>
+      </c>
+      <c r="B51" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="C51" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="D51" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="E51" s="10">
+        <v>6</v>
+      </c>
+      <c r="F51" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="G51" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="H51" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="I51" s="10"/>
+      <c r="J51" s="10"/>
+      <c r="K51" s="10"/>
+      <c r="L51" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="M51" s="10">
+        <v>1</v>
+      </c>
+      <c r="N51" s="10">
+        <v>1</v>
+      </c>
+      <c r="O51" s="10">
+        <v>850</v>
+      </c>
+      <c r="P51" s="10" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="10">
+        <v>50</v>
+      </c>
+      <c r="B52" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="C52" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="D52" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="E52" s="10">
+        <v>6</v>
+      </c>
+      <c r="F52" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="G52" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="H52" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="I52" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="J52" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="K52" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="L52" s="11"/>
+      <c r="M52" s="10">
+        <v>1</v>
+      </c>
+      <c r="N52" s="10">
+        <v>1</v>
+      </c>
+      <c r="O52" s="10">
+        <v>900</v>
+      </c>
+      <c r="P52" s="11"/>
+    </row>
+    <row r="53" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="10">
+        <v>51</v>
+      </c>
+      <c r="B53" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="C53" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="D53" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="E53" s="10">
+        <v>6</v>
+      </c>
+      <c r="F53" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="G53" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="H53" s="11" t="s">
+        <v>209</v>
+      </c>
+      <c r="I53" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="J53" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="K53" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="L53" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="M53" s="10">
+        <v>1</v>
+      </c>
+      <c r="N53" s="10">
+        <v>1</v>
+      </c>
+      <c r="O53" s="10">
+        <v>950</v>
+      </c>
+      <c r="P53" s="11" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="10">
+        <v>52</v>
+      </c>
+      <c r="B54" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="C54" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="D54" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="E54" s="10">
+        <v>6</v>
+      </c>
+      <c r="F54" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="G54" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="H54" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="I54" s="11"/>
+      <c r="J54" s="11"/>
+      <c r="K54" s="11"/>
+      <c r="L54" s="11" t="s">
+        <v>212</v>
+      </c>
+      <c r="M54" s="10">
+        <v>2</v>
+      </c>
+      <c r="N54" s="10">
+        <v>1</v>
+      </c>
+      <c r="O54" s="10">
+        <v>1000</v>
+      </c>
+      <c r="P54" s="11" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="10">
+        <v>53</v>
+      </c>
+      <c r="B55" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="C55" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="D55" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="E55" s="10">
+        <v>6</v>
+      </c>
+      <c r="F55" s="11" t="s">
+        <v>216</v>
+      </c>
+      <c r="G55" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="H55" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="I55" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="J55" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="K55" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="L55" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="M55" s="10">
+        <v>2</v>
+      </c>
+      <c r="N55" s="10">
+        <v>1</v>
+      </c>
+      <c r="O55" s="10">
+        <v>1050</v>
+      </c>
+      <c r="P55" s="10" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="10">
+        <v>54</v>
+      </c>
+      <c r="B56" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="C56" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="D56" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="E56" s="10">
+        <v>6</v>
+      </c>
+      <c r="F56" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="G56" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="H56" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="I56" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="J56" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="K56" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="L56" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="M56" s="10">
+        <v>2</v>
+      </c>
+      <c r="N56" s="10">
+        <v>1</v>
+      </c>
+      <c r="O56" s="10">
+        <v>1100</v>
+      </c>
+      <c r="P56" s="11" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="10">
+        <v>55</v>
+      </c>
+      <c r="B57" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="C57" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="D57" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="E57" s="10">
+        <v>6</v>
+      </c>
+      <c r="F57" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="G57" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="H57" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="I57" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="J57" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="K57" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="L57" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="M57" s="10">
+        <v>2</v>
+      </c>
+      <c r="N57" s="10">
+        <v>2</v>
+      </c>
+      <c r="O57" s="10">
+        <v>1200</v>
+      </c>
+      <c r="P57" s="11" t="s">
+        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar datos de desafíos (desafios.xlsx)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/desafios.xlsx
+++ b/public/resources/desafios.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2056CC57-C7A4-41FD-AD46-A059359AA68B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B5CB236-C9F4-44A3-BFB1-0DC9F6513F9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1068,7 +1068,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1128,6 +1128,33 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1529,8 +1556,8 @@
       <c r="N2" s="2">
         <v>0</v>
       </c>
-      <c r="O2" s="2">
-        <v>50</v>
+      <c r="O2" s="21">
+        <v>12</v>
       </c>
       <c r="P2" s="2"/>
     </row>
@@ -1565,8 +1592,8 @@
       <c r="N3" s="4">
         <v>0</v>
       </c>
-      <c r="O3" s="4">
-        <v>100</v>
+      <c r="O3" s="22">
+        <v>25</v>
       </c>
       <c r="P3" s="6" t="s">
         <v>15</v>
@@ -1613,8 +1640,8 @@
       <c r="N4" s="3">
         <v>0</v>
       </c>
-      <c r="O4" s="3">
-        <v>150</v>
+      <c r="O4" s="23">
+        <v>37</v>
       </c>
       <c r="P4" s="7"/>
     </row>
@@ -1655,8 +1682,8 @@
       <c r="N5" s="8">
         <v>0</v>
       </c>
-      <c r="O5" s="8">
-        <v>200</v>
+      <c r="O5" s="24">
+        <v>50</v>
       </c>
       <c r="P5" s="9" t="s">
         <v>48</v>
@@ -1693,8 +1720,8 @@
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
-      <c r="O6" s="2">
-        <v>200</v>
+      <c r="O6" s="21">
+        <v>50</v>
       </c>
       <c r="P6" s="2"/>
     </row>
@@ -1735,8 +1762,8 @@
       <c r="N7" s="4">
         <v>0</v>
       </c>
-      <c r="O7" s="4">
-        <v>250</v>
+      <c r="O7" s="22">
+        <v>62</v>
       </c>
       <c r="P7" s="4" t="s">
         <v>53</v>
@@ -1783,8 +1810,8 @@
       <c r="N8" s="3">
         <v>0</v>
       </c>
-      <c r="O8" s="3">
-        <v>300</v>
+      <c r="O8" s="23">
+        <v>75</v>
       </c>
       <c r="P8" s="6"/>
     </row>
@@ -1825,8 +1852,8 @@
       <c r="N9" s="8">
         <v>0</v>
       </c>
-      <c r="O9" s="8">
-        <v>350</v>
+      <c r="O9" s="24">
+        <v>87</v>
       </c>
       <c r="P9" s="9" t="s">
         <v>17</v>
@@ -1867,8 +1894,8 @@
       <c r="N10" s="2">
         <v>0</v>
       </c>
-      <c r="O10" s="2">
-        <v>350</v>
+      <c r="O10" s="21">
+        <v>87</v>
       </c>
       <c r="P10" s="2"/>
     </row>
@@ -1909,8 +1936,8 @@
       <c r="N11" s="4">
         <v>0</v>
       </c>
-      <c r="O11" s="4">
-        <v>400</v>
+      <c r="O11" s="22">
+        <v>100</v>
       </c>
       <c r="P11" s="6" t="s">
         <v>69</v>
@@ -1957,8 +1984,8 @@
       <c r="N12" s="3">
         <v>0</v>
       </c>
-      <c r="O12" s="3">
-        <v>450</v>
+      <c r="O12" s="23">
+        <v>112</v>
       </c>
       <c r="P12" s="7"/>
     </row>
@@ -1999,8 +2026,8 @@
       <c r="N13" s="8">
         <v>0</v>
       </c>
-      <c r="O13" s="8">
-        <v>500</v>
+      <c r="O13" s="24">
+        <v>125</v>
       </c>
       <c r="P13" s="9" t="s">
         <v>21</v>
@@ -2043,8 +2070,8 @@
       <c r="N14" s="2">
         <v>0</v>
       </c>
-      <c r="O14" s="2">
-        <v>500</v>
+      <c r="O14" s="21">
+        <v>125</v>
       </c>
       <c r="P14" s="2" t="s">
         <v>81</v>
@@ -2087,8 +2114,8 @@
       <c r="N15" s="4">
         <v>0</v>
       </c>
-      <c r="O15" s="4">
-        <v>550</v>
+      <c r="O15" s="22">
+        <v>137</v>
       </c>
       <c r="P15" s="4" t="s">
         <v>38</v>
@@ -2135,8 +2162,8 @@
       <c r="N16" s="3">
         <v>0</v>
       </c>
-      <c r="O16" s="3">
-        <v>600</v>
+      <c r="O16" s="23">
+        <v>150</v>
       </c>
       <c r="P16" s="7"/>
     </row>
@@ -2177,8 +2204,8 @@
       <c r="N17" s="8">
         <v>0</v>
       </c>
-      <c r="O17" s="8">
-        <v>650</v>
+      <c r="O17" s="24">
+        <v>162</v>
       </c>
       <c r="P17" s="9" t="s">
         <v>26</v>
@@ -2221,8 +2248,8 @@
       <c r="N18" s="2">
         <v>0</v>
       </c>
-      <c r="O18" s="2">
-        <v>650</v>
+      <c r="O18" s="21">
+        <v>162</v>
       </c>
       <c r="P18" s="2" t="s">
         <v>92</v>
@@ -2269,8 +2296,8 @@
       <c r="N19" s="4">
         <v>0</v>
       </c>
-      <c r="O19" s="4">
-        <v>700</v>
+      <c r="O19" s="22">
+        <v>175</v>
       </c>
       <c r="P19" s="4"/>
     </row>
@@ -2311,8 +2338,8 @@
       <c r="N20" s="3">
         <v>0</v>
       </c>
-      <c r="O20" s="3">
-        <v>750</v>
+      <c r="O20" s="23">
+        <v>187</v>
       </c>
       <c r="P20" s="7" t="s">
         <v>104</v>
@@ -2355,8 +2382,8 @@
       <c r="N21" s="8">
         <v>0</v>
       </c>
-      <c r="O21" s="8">
-        <v>800</v>
+      <c r="O21" s="24">
+        <v>200</v>
       </c>
       <c r="P21" s="9" t="s">
         <v>110</v>
@@ -2403,8 +2430,8 @@
       <c r="N22" s="10">
         <v>1</v>
       </c>
-      <c r="O22" s="10">
-        <v>800</v>
+      <c r="O22" s="25">
+        <v>200</v>
       </c>
       <c r="P22" s="10"/>
     </row>
@@ -2449,8 +2476,8 @@
       <c r="N23" s="10">
         <v>1</v>
       </c>
-      <c r="O23" s="10">
-        <v>850</v>
+      <c r="O23" s="25">
+        <v>212</v>
       </c>
       <c r="P23" s="10"/>
     </row>
@@ -2491,8 +2518,8 @@
       <c r="N24" s="10">
         <v>1</v>
       </c>
-      <c r="O24" s="10">
-        <v>900</v>
+      <c r="O24" s="25">
+        <v>225</v>
       </c>
       <c r="P24" s="11" t="s">
         <v>148</v>
@@ -2539,8 +2566,8 @@
       <c r="N25" s="10">
         <v>1</v>
       </c>
-      <c r="O25" s="10">
-        <v>950</v>
+      <c r="O25" s="25">
+        <v>237</v>
       </c>
       <c r="P25" s="11" t="s">
         <v>158</v>
@@ -2587,8 +2614,8 @@
       <c r="N26" s="10">
         <v>1</v>
       </c>
-      <c r="O26" s="10">
-        <v>1000</v>
+      <c r="O26" s="25">
+        <v>250</v>
       </c>
       <c r="P26" s="11"/>
     </row>
@@ -2633,8 +2660,8 @@
       <c r="N27" s="10">
         <v>1</v>
       </c>
-      <c r="O27" s="10">
-        <v>1050</v>
+      <c r="O27" s="25">
+        <v>262</v>
       </c>
       <c r="P27" s="10"/>
     </row>
@@ -2681,8 +2708,8 @@
       <c r="N28" s="10">
         <v>1</v>
       </c>
-      <c r="O28" s="10">
-        <v>1100</v>
+      <c r="O28" s="25">
+        <v>275</v>
       </c>
       <c r="P28" s="11" t="s">
         <v>124</v>
@@ -2731,8 +2758,8 @@
       <c r="N29" s="10">
         <v>2</v>
       </c>
-      <c r="O29" s="10">
-        <v>1200</v>
+      <c r="O29" s="25">
+        <v>300</v>
       </c>
       <c r="P29" s="11" t="s">
         <v>118</v>
@@ -2773,8 +2800,8 @@
       <c r="N30" s="12">
         <v>0</v>
       </c>
-      <c r="O30" s="12">
-        <v>50</v>
+      <c r="O30" s="26">
+        <v>12</v>
       </c>
       <c r="P30" s="12"/>
     </row>
@@ -2809,8 +2836,8 @@
       <c r="N31" s="14">
         <v>0</v>
       </c>
-      <c r="O31" s="14">
-        <v>100</v>
+      <c r="O31" s="27">
+        <v>25</v>
       </c>
       <c r="P31" s="15" t="s">
         <v>226</v>
@@ -2857,8 +2884,8 @@
       <c r="N32" s="16">
         <v>0</v>
       </c>
-      <c r="O32" s="16">
-        <v>150</v>
+      <c r="O32" s="28">
+        <v>37</v>
       </c>
       <c r="P32" s="17"/>
     </row>
@@ -2899,8 +2926,8 @@
       <c r="N33" s="18">
         <v>0</v>
       </c>
-      <c r="O33" s="18">
-        <v>200</v>
+      <c r="O33" s="29">
+        <v>50</v>
       </c>
       <c r="P33" s="19" t="s">
         <v>232</v>
@@ -2937,8 +2964,8 @@
       <c r="L34" s="12"/>
       <c r="M34" s="12"/>
       <c r="N34" s="12"/>
-      <c r="O34" s="12">
-        <v>200</v>
+      <c r="O34" s="26">
+        <v>50</v>
       </c>
       <c r="P34" s="12"/>
     </row>
@@ -2979,8 +3006,8 @@
       <c r="N35" s="14">
         <v>0</v>
       </c>
-      <c r="O35" s="14">
-        <v>250</v>
+      <c r="O35" s="27">
+        <v>62</v>
       </c>
       <c r="P35" s="15" t="s">
         <v>302</v>
@@ -3027,8 +3054,8 @@
       <c r="N36" s="16">
         <v>0</v>
       </c>
-      <c r="O36" s="16">
-        <v>300</v>
+      <c r="O36" s="28">
+        <v>75</v>
       </c>
       <c r="P36" s="17"/>
     </row>
@@ -3069,8 +3096,8 @@
       <c r="N37" s="18">
         <v>0</v>
       </c>
-      <c r="O37" s="18">
-        <v>350</v>
+      <c r="O37" s="29">
+        <v>87</v>
       </c>
       <c r="P37" s="19" t="s">
         <v>167</v>
@@ -3111,8 +3138,8 @@
       <c r="N38" s="12">
         <v>0</v>
       </c>
-      <c r="O38" s="12">
-        <v>350</v>
+      <c r="O38" s="26">
+        <v>87</v>
       </c>
       <c r="P38" s="12"/>
     </row>
@@ -3153,8 +3180,8 @@
       <c r="N39" s="14">
         <v>0</v>
       </c>
-      <c r="O39" s="14">
-        <v>400</v>
+      <c r="O39" s="27">
+        <v>100</v>
       </c>
       <c r="P39" s="15" t="s">
         <v>286</v>
@@ -3201,8 +3228,8 @@
       <c r="N40" s="16">
         <v>0</v>
       </c>
-      <c r="O40" s="16">
-        <v>450</v>
+      <c r="O40" s="28">
+        <v>112</v>
       </c>
       <c r="P40" s="17"/>
     </row>
@@ -3243,8 +3270,8 @@
       <c r="N41" s="18">
         <v>0</v>
       </c>
-      <c r="O41" s="18">
-        <v>500</v>
+      <c r="O41" s="29">
+        <v>125</v>
       </c>
       <c r="P41" s="19" t="s">
         <v>171</v>
@@ -3285,8 +3312,8 @@
       <c r="N42" s="12">
         <v>0</v>
       </c>
-      <c r="O42" s="12">
-        <v>500</v>
+      <c r="O42" s="26">
+        <v>125</v>
       </c>
       <c r="P42" s="12"/>
     </row>
@@ -3327,8 +3354,8 @@
       <c r="N43" s="14">
         <v>0</v>
       </c>
-      <c r="O43" s="14">
-        <v>550</v>
+      <c r="O43" s="27">
+        <v>137</v>
       </c>
       <c r="P43" s="15" t="s">
         <v>267</v>
@@ -3375,8 +3402,8 @@
       <c r="N44" s="16">
         <v>0</v>
       </c>
-      <c r="O44" s="16">
-        <v>600</v>
+      <c r="O44" s="28">
+        <v>150</v>
       </c>
       <c r="P44" s="17"/>
     </row>
@@ -3417,8 +3444,8 @@
       <c r="N45" s="18">
         <v>0</v>
       </c>
-      <c r="O45" s="18">
-        <v>650</v>
+      <c r="O45" s="29">
+        <v>162</v>
       </c>
       <c r="P45" s="19" t="s">
         <v>269</v>
@@ -3463,8 +3490,8 @@
       <c r="N46" s="12">
         <v>0</v>
       </c>
-      <c r="O46" s="12">
-        <v>650</v>
+      <c r="O46" s="26">
+        <v>162</v>
       </c>
       <c r="P46" s="12" t="s">
         <v>241</v>
@@ -3511,8 +3538,8 @@
       <c r="N47" s="14">
         <v>0</v>
       </c>
-      <c r="O47" s="14">
-        <v>700</v>
+      <c r="O47" s="27">
+        <v>175</v>
       </c>
       <c r="P47" s="15"/>
     </row>
@@ -3557,8 +3584,8 @@
       <c r="N48" s="16">
         <v>0</v>
       </c>
-      <c r="O48" s="16">
-        <v>750</v>
+      <c r="O48" s="28">
+        <v>187</v>
       </c>
       <c r="P48" s="17"/>
     </row>
@@ -3599,8 +3626,8 @@
       <c r="N49" s="18">
         <v>0</v>
       </c>
-      <c r="O49" s="18">
-        <v>800</v>
+      <c r="O49" s="29">
+        <v>200</v>
       </c>
       <c r="P49" s="19" t="s">
         <v>259</v>
@@ -3647,8 +3674,8 @@
       <c r="N50" s="10">
         <v>1</v>
       </c>
-      <c r="O50" s="10">
-        <v>800</v>
+      <c r="O50" s="25">
+        <v>200</v>
       </c>
       <c r="P50" s="10"/>
     </row>
@@ -3689,8 +3716,8 @@
       <c r="N51" s="10">
         <v>1</v>
       </c>
-      <c r="O51" s="10">
-        <v>850</v>
+      <c r="O51" s="25">
+        <v>212</v>
       </c>
       <c r="P51" s="10" t="s">
         <v>170</v>
@@ -3737,8 +3764,8 @@
       <c r="N52" s="10">
         <v>1</v>
       </c>
-      <c r="O52" s="10">
-        <v>900</v>
+      <c r="O52" s="25">
+        <v>225</v>
       </c>
       <c r="P52" s="11"/>
     </row>
@@ -3785,8 +3812,8 @@
       <c r="N53" s="10">
         <v>1</v>
       </c>
-      <c r="O53" s="10">
-        <v>950</v>
+      <c r="O53" s="25">
+        <v>237</v>
       </c>
       <c r="P53" s="11" t="s">
         <v>177</v>
@@ -3829,8 +3856,8 @@
       <c r="N54" s="10">
         <v>1</v>
       </c>
-      <c r="O54" s="10">
-        <v>1000</v>
+      <c r="O54" s="25">
+        <v>250</v>
       </c>
       <c r="P54" s="11" t="s">
         <v>212</v>
@@ -3879,8 +3906,8 @@
       <c r="N55" s="10">
         <v>1</v>
       </c>
-      <c r="O55" s="10">
-        <v>1050</v>
+      <c r="O55" s="25">
+        <v>262</v>
       </c>
       <c r="P55" s="10" t="s">
         <v>215</v>
@@ -3929,8 +3956,8 @@
       <c r="N56" s="10">
         <v>1</v>
       </c>
-      <c r="O56" s="10">
-        <v>1100</v>
+      <c r="O56" s="25">
+        <v>275</v>
       </c>
       <c r="P56" s="11" t="s">
         <v>168</v>
@@ -3979,8 +4006,8 @@
       <c r="N57" s="10">
         <v>2</v>
       </c>
-      <c r="O57" s="10">
-        <v>1200</v>
+      <c r="O57" s="25">
+        <v>300</v>
       </c>
       <c r="P57" s="11" t="s">
         <v>173</v>

</xml_diff>

<commit_message>
Align coop event panels, daily rewards at midnight, online missions, and mejorarCartas filters.
- Add shared eventoPanelUi for multijugador coop panels (carousel, rewards, difficulty picker).

- Reset daily envelope rewards at local midnight without stacking missed days.

- Replace pvp/evento_coop missions with online class; progress on completed PvP or coop event matches.

- Add search, affiliation, and power sort filters to all mejorarCartas tabs.

- Update mission/event Excel data and affiliation token icons.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/desafios.xlsx
+++ b/public/resources/desafios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37EC1F3D-AB7D-4940-B0DF-E978714450E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DCF96F0-F114-4D11-A433-872CD9EA6EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -720,9 +720,6 @@
     <t>Wonder Girl</t>
   </si>
   <si>
-    <t>Kid Flash</t>
-  </si>
-  <si>
     <t>Starfire</t>
   </si>
   <si>
@@ -958,6 +955,9 @@
   </si>
   <si>
     <t>tablero_background_gotham</t>
+  </si>
+  <si>
+    <t>Wally West</t>
   </si>
 </sst>
 </file>
@@ -1531,7 +1531,7 @@
         <v>23</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="P2" s="2"/>
       <c r="Q2" s="30" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1615,7 +1615,7 @@
         <v>15</v>
       </c>
       <c r="Q3" s="30" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="P4" s="7"/>
       <c r="Q4" s="30" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1711,7 +1711,7 @@
         <v>48</v>
       </c>
       <c r="Q5" s="30" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="P6" s="2"/>
       <c r="Q6" s="30" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1797,7 +1797,7 @@
         <v>53</v>
       </c>
       <c r="Q7" s="30" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1846,7 +1846,7 @@
       </c>
       <c r="P8" s="6"/>
       <c r="Q8" s="30" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="9" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1893,7 +1893,7 @@
         <v>17</v>
       </c>
       <c r="Q9" s="30" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="10" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2925,13 +2925,13 @@
         <v>225</v>
       </c>
       <c r="H32" s="17" t="s">
-        <v>231</v>
+        <v>310</v>
       </c>
       <c r="I32" s="17" t="s">
         <v>226</v>
       </c>
       <c r="J32" s="17" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="K32" s="17" t="s">
         <v>218</v>
@@ -2960,7 +2960,7 @@
         <v>222</v>
       </c>
       <c r="D33" s="18" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E33" s="18">
         <v>1</v>
@@ -2972,13 +2972,13 @@
         <v>226</v>
       </c>
       <c r="H33" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="I33" s="19"/>
       <c r="J33" s="19"/>
       <c r="K33" s="19"/>
       <c r="L33" s="19" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="M33" s="18">
         <v>1</v>
@@ -2990,7 +2990,7 @@
         <v>50</v>
       </c>
       <c r="P33" s="19" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="Q33" s="30"/>
     </row>
@@ -3002,22 +3002,22 @@
         <v>164</v>
       </c>
       <c r="C34" s="12" t="s">
+        <v>292</v>
+      </c>
+      <c r="D34" s="12" t="s">
         <v>293</v>
-      </c>
-      <c r="D34" s="12" t="s">
-        <v>294</v>
       </c>
       <c r="E34" s="12">
         <v>2</v>
       </c>
       <c r="F34" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="G34" s="13" t="s">
         <v>295</v>
       </c>
-      <c r="G34" s="13" t="s">
+      <c r="H34" s="13" t="s">
         <v>296</v>
-      </c>
-      <c r="H34" s="13" t="s">
-        <v>297</v>
       </c>
       <c r="I34" s="12"/>
       <c r="J34" s="12"/>
@@ -3039,28 +3039,28 @@
         <v>164</v>
       </c>
       <c r="C35" s="14" t="s">
+        <v>297</v>
+      </c>
+      <c r="D35" s="14" t="s">
         <v>298</v>
-      </c>
-      <c r="D35" s="14" t="s">
-        <v>299</v>
       </c>
       <c r="E35" s="14">
         <v>2</v>
       </c>
       <c r="F35" s="15" t="s">
+        <v>299</v>
+      </c>
+      <c r="G35" s="15" t="s">
+        <v>233</v>
+      </c>
+      <c r="H35" s="15" t="s">
         <v>300</v>
-      </c>
-      <c r="G35" s="15" t="s">
-        <v>234</v>
-      </c>
-      <c r="H35" s="15" t="s">
-        <v>301</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="14"/>
       <c r="K35" s="14"/>
       <c r="L35" s="15" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="M35" s="14">
         <v>0</v>
@@ -3072,7 +3072,7 @@
         <v>62</v>
       </c>
       <c r="P35" s="15" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="Q35" s="30"/>
     </row>
@@ -3084,28 +3084,28 @@
         <v>164</v>
       </c>
       <c r="C36" s="16" t="s">
+        <v>302</v>
+      </c>
+      <c r="D36" s="16" t="s">
         <v>303</v>
-      </c>
-      <c r="D36" s="16" t="s">
-        <v>304</v>
       </c>
       <c r="E36" s="16">
         <v>2</v>
       </c>
       <c r="F36" s="17" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G36" s="17" t="s">
+        <v>300</v>
+      </c>
+      <c r="H36" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="I36" s="17" t="s">
         <v>301</v>
       </c>
-      <c r="H36" s="17" t="s">
-        <v>234</v>
-      </c>
-      <c r="I36" s="17" t="s">
-        <v>302</v>
-      </c>
       <c r="J36" s="17" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="K36" s="17" t="s">
         <v>167</v>
@@ -3131,22 +3131,22 @@
         <v>164</v>
       </c>
       <c r="C37" s="18" t="s">
+        <v>305</v>
+      </c>
+      <c r="D37" s="18" t="s">
         <v>306</v>
-      </c>
-      <c r="D37" s="18" t="s">
-        <v>307</v>
       </c>
       <c r="E37" s="18">
         <v>2</v>
       </c>
       <c r="F37" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G37" s="19" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H37" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="I37" s="19"/>
       <c r="J37" s="19"/>
@@ -3176,22 +3176,22 @@
         <v>164</v>
       </c>
       <c r="C38" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="D38" s="12" t="s">
         <v>276</v>
-      </c>
-      <c r="D38" s="12" t="s">
-        <v>277</v>
       </c>
       <c r="E38" s="12">
         <v>3</v>
       </c>
       <c r="F38" s="13" t="s">
+        <v>277</v>
+      </c>
+      <c r="G38" s="13" t="s">
         <v>278</v>
       </c>
-      <c r="G38" s="13" t="s">
+      <c r="H38" s="13" t="s">
         <v>279</v>
-      </c>
-      <c r="H38" s="13" t="s">
-        <v>280</v>
       </c>
       <c r="I38" s="12"/>
       <c r="J38" s="12"/>
@@ -3217,28 +3217,28 @@
         <v>164</v>
       </c>
       <c r="C39" s="14" t="s">
+        <v>280</v>
+      </c>
+      <c r="D39" s="14" t="s">
         <v>281</v>
-      </c>
-      <c r="D39" s="14" t="s">
-        <v>282</v>
       </c>
       <c r="E39" s="14">
         <v>3</v>
       </c>
       <c r="F39" s="15" t="s">
+        <v>282</v>
+      </c>
+      <c r="G39" s="15" t="s">
         <v>283</v>
       </c>
-      <c r="G39" s="15" t="s">
+      <c r="H39" s="15" t="s">
         <v>284</v>
-      </c>
-      <c r="H39" s="15" t="s">
-        <v>285</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="14"/>
       <c r="K39" s="14"/>
       <c r="L39" s="15" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="M39" s="14">
         <v>0</v>
@@ -3250,7 +3250,7 @@
         <v>100</v>
       </c>
       <c r="P39" s="15" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="Q39" s="30"/>
     </row>
@@ -3262,28 +3262,28 @@
         <v>164</v>
       </c>
       <c r="C40" s="16" t="s">
+        <v>286</v>
+      </c>
+      <c r="D40" s="16" t="s">
         <v>287</v>
-      </c>
-      <c r="D40" s="16" t="s">
-        <v>288</v>
       </c>
       <c r="E40" s="16">
         <v>3</v>
       </c>
       <c r="F40" s="17" t="s">
+        <v>288</v>
+      </c>
+      <c r="G40" s="17" t="s">
+        <v>282</v>
+      </c>
+      <c r="H40" s="17" t="s">
+        <v>277</v>
+      </c>
+      <c r="I40" s="17" t="s">
         <v>289</v>
       </c>
-      <c r="G40" s="17" t="s">
-        <v>283</v>
-      </c>
-      <c r="H40" s="17" t="s">
-        <v>278</v>
-      </c>
-      <c r="I40" s="17" t="s">
-        <v>290</v>
-      </c>
       <c r="J40" s="17" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K40" s="17" t="s">
         <v>171</v>
@@ -3309,22 +3309,22 @@
         <v>164</v>
       </c>
       <c r="C41" s="18" t="s">
+        <v>290</v>
+      </c>
+      <c r="D41" s="18" t="s">
         <v>291</v>
-      </c>
-      <c r="D41" s="18" t="s">
-        <v>292</v>
       </c>
       <c r="E41" s="18">
         <v>3</v>
       </c>
       <c r="F41" s="19" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G41" s="19" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="H41" s="19" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="I41" s="19"/>
       <c r="J41" s="19"/>
@@ -3354,22 +3354,22 @@
         <v>164</v>
       </c>
       <c r="C42" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="D42" s="12" t="s">
         <v>260</v>
-      </c>
-      <c r="D42" s="12" t="s">
-        <v>261</v>
       </c>
       <c r="E42" s="12">
         <v>4</v>
       </c>
       <c r="F42" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="G42" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="G42" s="13" t="s">
+      <c r="H42" s="13" t="s">
         <v>263</v>
-      </c>
-      <c r="H42" s="13" t="s">
-        <v>264</v>
       </c>
       <c r="I42" s="12"/>
       <c r="J42" s="12"/>
@@ -3395,28 +3395,28 @@
         <v>164</v>
       </c>
       <c r="C43" s="14" t="s">
+        <v>264</v>
+      </c>
+      <c r="D43" s="14" t="s">
         <v>265</v>
-      </c>
-      <c r="D43" s="14" t="s">
-        <v>266</v>
       </c>
       <c r="E43" s="14">
         <v>4</v>
       </c>
       <c r="F43" s="15" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G43" s="15" t="s">
         <v>226</v>
       </c>
       <c r="H43" s="15" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="I43" s="14"/>
       <c r="J43" s="14"/>
       <c r="K43" s="14"/>
       <c r="L43" s="15" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="M43" s="14">
         <v>0</v>
@@ -3428,7 +3428,7 @@
         <v>137</v>
       </c>
       <c r="P43" s="15" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="Q43" s="30"/>
     </row>
@@ -3440,31 +3440,31 @@
         <v>164</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E44" s="16">
         <v>4</v>
       </c>
       <c r="F44" s="17" t="s">
+        <v>262</v>
+      </c>
+      <c r="G44" s="17" t="s">
         <v>263</v>
       </c>
-      <c r="G44" s="17" t="s">
-        <v>264</v>
-      </c>
       <c r="H44" s="17" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I44" s="17" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="J44" s="17" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="K44" s="17" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="L44" s="17"/>
       <c r="M44" s="16">
@@ -3487,28 +3487,28 @@
         <v>164</v>
       </c>
       <c r="C45" s="18" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D45" s="18" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E45" s="18">
         <v>4</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G45" s="19" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="H45" s="19" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="I45" s="19"/>
       <c r="J45" s="19"/>
       <c r="K45" s="19"/>
       <c r="L45" s="19" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="M45" s="18">
         <v>1</v>
@@ -3520,7 +3520,7 @@
         <v>162</v>
       </c>
       <c r="P45" s="19" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="Q45" s="30"/>
     </row>
@@ -3532,30 +3532,30 @@
         <v>164</v>
       </c>
       <c r="C46" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="D46" s="12" t="s">
         <v>235</v>
-      </c>
-      <c r="D46" s="12" t="s">
-        <v>236</v>
       </c>
       <c r="E46" s="12">
         <v>5</v>
       </c>
       <c r="F46" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="G46" s="13" t="s">
         <v>237</v>
       </c>
-      <c r="G46" s="13" t="s">
+      <c r="H46" s="13" t="s">
         <v>238</v>
       </c>
-      <c r="H46" s="13" t="s">
+      <c r="I46" s="12" t="s">
         <v>239</v>
-      </c>
-      <c r="I46" s="12" t="s">
-        <v>240</v>
       </c>
       <c r="J46" s="12"/>
       <c r="K46" s="12"/>
       <c r="L46" s="12" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="M46" s="12">
         <v>0</v>
@@ -3567,7 +3567,7 @@
         <v>162</v>
       </c>
       <c r="P46" s="12" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="Q46" s="30"/>
     </row>
@@ -3579,22 +3579,22 @@
         <v>164</v>
       </c>
       <c r="C47" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="D47" s="14" t="s">
         <v>242</v>
-      </c>
-      <c r="D47" s="14" t="s">
-        <v>243</v>
       </c>
       <c r="E47" s="14">
         <v>5</v>
       </c>
       <c r="F47" s="15" t="s">
+        <v>243</v>
+      </c>
+      <c r="G47" s="15" t="s">
         <v>244</v>
       </c>
-      <c r="G47" s="15" t="s">
+      <c r="H47" s="15" t="s">
         <v>245</v>
-      </c>
-      <c r="H47" s="15" t="s">
-        <v>246</v>
       </c>
       <c r="I47" s="14" t="s">
         <v>230</v>
@@ -3603,7 +3603,7 @@
         <v>225</v>
       </c>
       <c r="K47" s="14" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="L47" s="15"/>
       <c r="M47" s="14">
@@ -3626,31 +3626,31 @@
         <v>164</v>
       </c>
       <c r="C48" s="16" t="s">
+        <v>247</v>
+      </c>
+      <c r="D48" s="16" t="s">
         <v>248</v>
-      </c>
-      <c r="D48" s="16" t="s">
-        <v>249</v>
       </c>
       <c r="E48" s="16">
         <v>5</v>
       </c>
       <c r="F48" s="17" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G48" s="17" t="s">
         <v>206</v>
       </c>
       <c r="H48" s="17" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I48" s="17" t="s">
         <v>203</v>
       </c>
       <c r="J48" s="17" t="s">
+        <v>250</v>
+      </c>
+      <c r="K48" s="17" t="s">
         <v>251</v>
-      </c>
-      <c r="K48" s="17" t="s">
-        <v>252</v>
       </c>
       <c r="L48" s="17"/>
       <c r="M48" s="16">
@@ -3673,28 +3673,28 @@
         <v>164</v>
       </c>
       <c r="C49" s="18" t="s">
+        <v>253</v>
+      </c>
+      <c r="D49" s="18" t="s">
         <v>254</v>
-      </c>
-      <c r="D49" s="18" t="s">
-        <v>255</v>
       </c>
       <c r="E49" s="18">
         <v>5</v>
       </c>
       <c r="F49" s="19" t="s">
+        <v>255</v>
+      </c>
+      <c r="G49" s="19" t="s">
         <v>256</v>
       </c>
-      <c r="G49" s="19" t="s">
+      <c r="H49" s="19" t="s">
         <v>257</v>
-      </c>
-      <c r="H49" s="19" t="s">
-        <v>258</v>
       </c>
       <c r="I49" s="19"/>
       <c r="J49" s="19"/>
       <c r="K49" s="19"/>
       <c r="L49" s="19" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="M49" s="18">
         <v>1</v>
@@ -3706,7 +3706,7 @@
         <v>200</v>
       </c>
       <c r="P49" s="19" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="Q49" s="30"/>
     </row>

</xml_diff>

<commit_message>
Release 1.2.6: skill_class filters, online mission tracking fix, and collection polish.
EOF

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/desafios.xlsx
+++ b/public/resources/desafios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DCF96F0-F114-4D11-A433-872CD9EA6EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA5DA75D-466E-448D-B835-763C7EC69F36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -513,9 +513,6 @@
     <t>Weasel</t>
   </si>
   <si>
-    <t>Boodsport</t>
-  </si>
-  <si>
     <t>King Shark</t>
   </si>
   <si>
@@ -958,6 +955,9 @@
   </si>
   <si>
     <t>Wally West</t>
+  </si>
+  <si>
+    <t>Bloodspot</t>
   </si>
 </sst>
 </file>
@@ -1531,7 +1531,7 @@
         <v>23</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="P2" s="2"/>
       <c r="Q2" s="30" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1615,7 +1615,7 @@
         <v>15</v>
       </c>
       <c r="Q3" s="30" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="P4" s="7"/>
       <c r="Q4" s="30" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1711,7 +1711,7 @@
         <v>48</v>
       </c>
       <c r="Q5" s="30" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="P6" s="2"/>
       <c r="Q6" s="30" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1797,7 +1797,7 @@
         <v>53</v>
       </c>
       <c r="Q7" s="30" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1846,7 +1846,7 @@
       </c>
       <c r="P8" s="6"/>
       <c r="Q8" s="30" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="9" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1893,7 +1893,7 @@
         <v>17</v>
       </c>
       <c r="Q9" s="30" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="10" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2461,10 +2461,10 @@
         <v>161</v>
       </c>
       <c r="H22" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="I22" s="10" t="s">
         <v>162</v>
-      </c>
-      <c r="I22" s="10" t="s">
-        <v>163</v>
       </c>
       <c r="J22" s="10" t="s">
         <v>103</v>
@@ -2827,25 +2827,25 @@
         <v>28</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E30" s="12">
         <v>1</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G30" s="13" t="s">
+        <v>224</v>
+      </c>
+      <c r="H30" s="13" t="s">
         <v>225</v>
-      </c>
-      <c r="H30" s="13" t="s">
-        <v>226</v>
       </c>
       <c r="I30" s="12"/>
       <c r="J30" s="12"/>
@@ -2868,13 +2868,13 @@
         <v>29</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C31" s="14" t="s">
+        <v>226</v>
+      </c>
+      <c r="D31" s="14" t="s">
         <v>227</v>
-      </c>
-      <c r="D31" s="14" t="s">
-        <v>228</v>
       </c>
       <c r="E31" s="14">
         <v>1</v>
@@ -2886,7 +2886,7 @@
       <c r="J31" s="14"/>
       <c r="K31" s="14"/>
       <c r="L31" s="15" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="M31" s="14">
         <v>0</v>
@@ -2898,7 +2898,7 @@
         <v>25</v>
       </c>
       <c r="P31" s="15" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="Q31" s="30"/>
     </row>
@@ -2907,34 +2907,34 @@
         <v>30</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C32" s="18" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E32" s="16">
         <v>1</v>
       </c>
       <c r="F32" s="17" t="s">
+        <v>229</v>
+      </c>
+      <c r="G32" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="H32" s="17" t="s">
+        <v>309</v>
+      </c>
+      <c r="I32" s="17" t="s">
+        <v>225</v>
+      </c>
+      <c r="J32" s="17" t="s">
         <v>230</v>
       </c>
-      <c r="G32" s="17" t="s">
-        <v>225</v>
-      </c>
-      <c r="H32" s="17" t="s">
-        <v>310</v>
-      </c>
-      <c r="I32" s="17" t="s">
-        <v>226</v>
-      </c>
-      <c r="J32" s="17" t="s">
-        <v>231</v>
-      </c>
       <c r="K32" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="L32" s="17"/>
       <c r="M32" s="16">
@@ -2954,31 +2954,31 @@
         <v>31</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C33" s="18" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D33" s="18" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E33" s="18">
         <v>1</v>
       </c>
       <c r="F33" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="G33" s="19" t="s">
         <v>225</v>
       </c>
-      <c r="G33" s="19" t="s">
-        <v>226</v>
-      </c>
       <c r="H33" s="19" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="I33" s="19"/>
       <c r="J33" s="19"/>
       <c r="K33" s="19"/>
       <c r="L33" s="19" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="M33" s="18">
         <v>1</v>
@@ -2990,7 +2990,7 @@
         <v>50</v>
       </c>
       <c r="P33" s="19" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="Q33" s="30"/>
     </row>
@@ -2999,25 +2999,25 @@
         <v>32</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C34" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="D34" s="12" t="s">
         <v>292</v>
-      </c>
-      <c r="D34" s="12" t="s">
-        <v>293</v>
       </c>
       <c r="E34" s="12">
         <v>2</v>
       </c>
       <c r="F34" s="13" t="s">
+        <v>293</v>
+      </c>
+      <c r="G34" s="13" t="s">
         <v>294</v>
       </c>
-      <c r="G34" s="13" t="s">
+      <c r="H34" s="13" t="s">
         <v>295</v>
-      </c>
-      <c r="H34" s="13" t="s">
-        <v>296</v>
       </c>
       <c r="I34" s="12"/>
       <c r="J34" s="12"/>
@@ -3036,31 +3036,31 @@
         <v>33</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C35" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="D35" s="14" t="s">
         <v>297</v>
-      </c>
-      <c r="D35" s="14" t="s">
-        <v>298</v>
       </c>
       <c r="E35" s="14">
         <v>2</v>
       </c>
       <c r="F35" s="15" t="s">
+        <v>298</v>
+      </c>
+      <c r="G35" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="H35" s="15" t="s">
         <v>299</v>
-      </c>
-      <c r="G35" s="15" t="s">
-        <v>233</v>
-      </c>
-      <c r="H35" s="15" t="s">
-        <v>300</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="14"/>
       <c r="K35" s="14"/>
       <c r="L35" s="15" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="M35" s="14">
         <v>0</v>
@@ -3072,7 +3072,7 @@
         <v>62</v>
       </c>
       <c r="P35" s="15" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="Q35" s="30"/>
     </row>
@@ -3081,34 +3081,34 @@
         <v>34</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C36" s="16" t="s">
+        <v>301</v>
+      </c>
+      <c r="D36" s="16" t="s">
         <v>302</v>
-      </c>
-      <c r="D36" s="16" t="s">
-        <v>303</v>
       </c>
       <c r="E36" s="16">
         <v>2</v>
       </c>
       <c r="F36" s="17" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G36" s="17" t="s">
+        <v>299</v>
+      </c>
+      <c r="H36" s="17" t="s">
+        <v>232</v>
+      </c>
+      <c r="I36" s="17" t="s">
         <v>300</v>
       </c>
-      <c r="H36" s="17" t="s">
-        <v>233</v>
-      </c>
-      <c r="I36" s="17" t="s">
-        <v>301</v>
-      </c>
       <c r="J36" s="17" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K36" s="17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="L36" s="17"/>
       <c r="M36" s="16">
@@ -3128,31 +3128,31 @@
         <v>35</v>
       </c>
       <c r="B37" s="18" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C37" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="D37" s="18" t="s">
         <v>305</v>
-      </c>
-      <c r="D37" s="18" t="s">
-        <v>306</v>
       </c>
       <c r="E37" s="18">
         <v>2</v>
       </c>
       <c r="F37" s="19" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G37" s="19" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H37" s="19" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="I37" s="19"/>
       <c r="J37" s="19"/>
       <c r="K37" s="19"/>
       <c r="L37" s="19" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="M37" s="18">
         <v>1</v>
@@ -3164,7 +3164,7 @@
         <v>87</v>
       </c>
       <c r="P37" s="19" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="Q37" s="30"/>
     </row>
@@ -3173,25 +3173,25 @@
         <v>36</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C38" s="12" t="s">
+        <v>274</v>
+      </c>
+      <c r="D38" s="12" t="s">
         <v>275</v>
-      </c>
-      <c r="D38" s="12" t="s">
-        <v>276</v>
       </c>
       <c r="E38" s="12">
         <v>3</v>
       </c>
       <c r="F38" s="13" t="s">
+        <v>276</v>
+      </c>
+      <c r="G38" s="13" t="s">
         <v>277</v>
       </c>
-      <c r="G38" s="13" t="s">
+      <c r="H38" s="13" t="s">
         <v>278</v>
-      </c>
-      <c r="H38" s="13" t="s">
-        <v>279</v>
       </c>
       <c r="I38" s="12"/>
       <c r="J38" s="12"/>
@@ -3214,31 +3214,31 @@
         <v>37</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C39" s="14" t="s">
+        <v>279</v>
+      </c>
+      <c r="D39" s="14" t="s">
         <v>280</v>
-      </c>
-      <c r="D39" s="14" t="s">
-        <v>281</v>
       </c>
       <c r="E39" s="14">
         <v>3</v>
       </c>
       <c r="F39" s="15" t="s">
+        <v>281</v>
+      </c>
+      <c r="G39" s="15" t="s">
         <v>282</v>
       </c>
-      <c r="G39" s="15" t="s">
+      <c r="H39" s="15" t="s">
         <v>283</v>
-      </c>
-      <c r="H39" s="15" t="s">
-        <v>284</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="14"/>
       <c r="K39" s="14"/>
       <c r="L39" s="15" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="M39" s="14">
         <v>0</v>
@@ -3250,7 +3250,7 @@
         <v>100</v>
       </c>
       <c r="P39" s="15" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="Q39" s="30"/>
     </row>
@@ -3259,34 +3259,34 @@
         <v>38</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C40" s="16" t="s">
+        <v>285</v>
+      </c>
+      <c r="D40" s="16" t="s">
         <v>286</v>
-      </c>
-      <c r="D40" s="16" t="s">
-        <v>287</v>
       </c>
       <c r="E40" s="16">
         <v>3</v>
       </c>
       <c r="F40" s="17" t="s">
+        <v>287</v>
+      </c>
+      <c r="G40" s="17" t="s">
+        <v>281</v>
+      </c>
+      <c r="H40" s="17" t="s">
+        <v>276</v>
+      </c>
+      <c r="I40" s="17" t="s">
         <v>288</v>
       </c>
-      <c r="G40" s="17" t="s">
-        <v>282</v>
-      </c>
-      <c r="H40" s="17" t="s">
-        <v>277</v>
-      </c>
-      <c r="I40" s="17" t="s">
-        <v>289</v>
-      </c>
       <c r="J40" s="17" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K40" s="17" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="L40" s="17"/>
       <c r="M40" s="16">
@@ -3306,31 +3306,31 @@
         <v>39</v>
       </c>
       <c r="B41" s="18" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C41" s="18" t="s">
+        <v>289</v>
+      </c>
+      <c r="D41" s="18" t="s">
         <v>290</v>
-      </c>
-      <c r="D41" s="18" t="s">
-        <v>291</v>
       </c>
       <c r="E41" s="18">
         <v>3</v>
       </c>
       <c r="F41" s="19" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G41" s="19" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="H41" s="19" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="I41" s="19"/>
       <c r="J41" s="19"/>
       <c r="K41" s="19"/>
       <c r="L41" s="19" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="M41" s="18">
         <v>1</v>
@@ -3342,7 +3342,7 @@
         <v>125</v>
       </c>
       <c r="P41" s="19" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="Q41" s="30"/>
     </row>
@@ -3351,25 +3351,25 @@
         <v>40</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C42" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="D42" s="12" t="s">
         <v>259</v>
-      </c>
-      <c r="D42" s="12" t="s">
-        <v>260</v>
       </c>
       <c r="E42" s="12">
         <v>4</v>
       </c>
       <c r="F42" s="13" t="s">
+        <v>260</v>
+      </c>
+      <c r="G42" s="13" t="s">
         <v>261</v>
       </c>
-      <c r="G42" s="13" t="s">
+      <c r="H42" s="13" t="s">
         <v>262</v>
-      </c>
-      <c r="H42" s="13" t="s">
-        <v>263</v>
       </c>
       <c r="I42" s="12"/>
       <c r="J42" s="12"/>
@@ -3392,31 +3392,31 @@
         <v>41</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C43" s="14" t="s">
+        <v>263</v>
+      </c>
+      <c r="D43" s="14" t="s">
         <v>264</v>
-      </c>
-      <c r="D43" s="14" t="s">
-        <v>265</v>
       </c>
       <c r="E43" s="14">
         <v>4</v>
       </c>
       <c r="F43" s="15" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H43" s="15" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="I43" s="14"/>
       <c r="J43" s="14"/>
       <c r="K43" s="14"/>
       <c r="L43" s="15" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="M43" s="14">
         <v>0</v>
@@ -3428,7 +3428,7 @@
         <v>137</v>
       </c>
       <c r="P43" s="15" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="Q43" s="30"/>
     </row>
@@ -3437,34 +3437,34 @@
         <v>42</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E44" s="16">
         <v>4</v>
       </c>
       <c r="F44" s="17" t="s">
+        <v>261</v>
+      </c>
+      <c r="G44" s="17" t="s">
         <v>262</v>
       </c>
-      <c r="G44" s="17" t="s">
-        <v>263</v>
-      </c>
       <c r="H44" s="17" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I44" s="17" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="J44" s="17" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="K44" s="17" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="L44" s="17"/>
       <c r="M44" s="16">
@@ -3484,31 +3484,31 @@
         <v>43</v>
       </c>
       <c r="B45" s="18" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C45" s="18" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D45" s="18" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E45" s="18">
         <v>4</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G45" s="19" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="H45" s="19" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="I45" s="19"/>
       <c r="J45" s="19"/>
       <c r="K45" s="19"/>
       <c r="L45" s="19" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="M45" s="18">
         <v>1</v>
@@ -3520,7 +3520,7 @@
         <v>162</v>
       </c>
       <c r="P45" s="19" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="Q45" s="30"/>
     </row>
@@ -3529,33 +3529,33 @@
         <v>44</v>
       </c>
       <c r="B46" s="12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C46" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="D46" s="12" t="s">
         <v>234</v>
-      </c>
-      <c r="D46" s="12" t="s">
-        <v>235</v>
       </c>
       <c r="E46" s="12">
         <v>5</v>
       </c>
       <c r="F46" s="13" t="s">
+        <v>235</v>
+      </c>
+      <c r="G46" s="13" t="s">
         <v>236</v>
       </c>
-      <c r="G46" s="13" t="s">
+      <c r="H46" s="13" t="s">
         <v>237</v>
       </c>
-      <c r="H46" s="13" t="s">
+      <c r="I46" s="12" t="s">
         <v>238</v>
-      </c>
-      <c r="I46" s="12" t="s">
-        <v>239</v>
       </c>
       <c r="J46" s="12"/>
       <c r="K46" s="12"/>
       <c r="L46" s="12" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="M46" s="12">
         <v>0</v>
@@ -3567,7 +3567,7 @@
         <v>162</v>
       </c>
       <c r="P46" s="12" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="Q46" s="30"/>
     </row>
@@ -3576,34 +3576,34 @@
         <v>45</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C47" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="D47" s="14" t="s">
         <v>241</v>
-      </c>
-      <c r="D47" s="14" t="s">
-        <v>242</v>
       </c>
       <c r="E47" s="14">
         <v>5</v>
       </c>
       <c r="F47" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="G47" s="15" t="s">
         <v>243</v>
       </c>
-      <c r="G47" s="15" t="s">
+      <c r="H47" s="15" t="s">
         <v>244</v>
       </c>
-      <c r="H47" s="15" t="s">
+      <c r="I47" s="14" t="s">
+        <v>229</v>
+      </c>
+      <c r="J47" s="14" t="s">
+        <v>224</v>
+      </c>
+      <c r="K47" s="14" t="s">
         <v>245</v>
-      </c>
-      <c r="I47" s="14" t="s">
-        <v>230</v>
-      </c>
-      <c r="J47" s="14" t="s">
-        <v>225</v>
-      </c>
-      <c r="K47" s="14" t="s">
-        <v>246</v>
       </c>
       <c r="L47" s="15"/>
       <c r="M47" s="14">
@@ -3623,34 +3623,34 @@
         <v>46</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C48" s="16" t="s">
+        <v>246</v>
+      </c>
+      <c r="D48" s="16" t="s">
         <v>247</v>
-      </c>
-      <c r="D48" s="16" t="s">
-        <v>248</v>
       </c>
       <c r="E48" s="16">
         <v>5</v>
       </c>
       <c r="F48" s="17" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G48" s="17" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H48" s="17" t="s">
+        <v>248</v>
+      </c>
+      <c r="I48" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="J48" s="17" t="s">
         <v>249</v>
       </c>
-      <c r="I48" s="17" t="s">
-        <v>203</v>
-      </c>
-      <c r="J48" s="17" t="s">
+      <c r="K48" s="17" t="s">
         <v>250</v>
-      </c>
-      <c r="K48" s="17" t="s">
-        <v>251</v>
       </c>
       <c r="L48" s="17"/>
       <c r="M48" s="16">
@@ -3670,31 +3670,31 @@
         <v>47</v>
       </c>
       <c r="B49" s="18" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C49" s="18" t="s">
+        <v>252</v>
+      </c>
+      <c r="D49" s="18" t="s">
         <v>253</v>
-      </c>
-      <c r="D49" s="18" t="s">
-        <v>254</v>
       </c>
       <c r="E49" s="18">
         <v>5</v>
       </c>
       <c r="F49" s="19" t="s">
+        <v>254</v>
+      </c>
+      <c r="G49" s="19" t="s">
         <v>255</v>
       </c>
-      <c r="G49" s="19" t="s">
+      <c r="H49" s="19" t="s">
         <v>256</v>
-      </c>
-      <c r="H49" s="19" t="s">
-        <v>257</v>
       </c>
       <c r="I49" s="19"/>
       <c r="J49" s="19"/>
       <c r="K49" s="19"/>
       <c r="L49" s="19" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="M49" s="18">
         <v>1</v>
@@ -3706,7 +3706,7 @@
         <v>200</v>
       </c>
       <c r="P49" s="19" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="Q49" s="30"/>
     </row>
@@ -3715,34 +3715,34 @@
         <v>48</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C50" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="D50" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="D50" s="10" t="s">
-        <v>181</v>
       </c>
       <c r="E50" s="10">
         <v>6</v>
       </c>
       <c r="F50" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="G50" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="G50" s="10" t="s">
+      <c r="H50" s="10" t="s">
         <v>183</v>
       </c>
-      <c r="H50" s="10" t="s">
+      <c r="I50" s="10" t="s">
         <v>184</v>
       </c>
-      <c r="I50" s="10" t="s">
+      <c r="J50" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="J50" s="10" t="s">
-        <v>186</v>
-      </c>
       <c r="K50" s="10" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="L50" s="10"/>
       <c r="M50" s="10">
@@ -3762,31 +3762,31 @@
         <v>49</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C51" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="D51" s="10" t="s">
         <v>187</v>
-      </c>
-      <c r="D51" s="10" t="s">
-        <v>188</v>
       </c>
       <c r="E51" s="10">
         <v>6</v>
       </c>
       <c r="F51" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="G51" s="11" t="s">
         <v>189</v>
       </c>
-      <c r="G51" s="11" t="s">
+      <c r="H51" s="11" t="s">
         <v>190</v>
-      </c>
-      <c r="H51" s="11" t="s">
-        <v>191</v>
       </c>
       <c r="I51" s="10"/>
       <c r="J51" s="10"/>
       <c r="K51" s="10"/>
       <c r="L51" s="10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="M51" s="10">
         <v>1</v>
@@ -3798,7 +3798,7 @@
         <v>212</v>
       </c>
       <c r="P51" s="10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="Q51" s="30"/>
     </row>
@@ -3807,34 +3807,34 @@
         <v>50</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C52" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="D52" s="10" t="s">
         <v>192</v>
-      </c>
-      <c r="D52" s="10" t="s">
-        <v>193</v>
       </c>
       <c r="E52" s="10">
         <v>6</v>
       </c>
       <c r="F52" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="G52" s="11" t="s">
         <v>194</v>
       </c>
-      <c r="G52" s="11" t="s">
+      <c r="H52" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="H52" s="11" t="s">
+      <c r="I52" s="11" t="s">
         <v>196</v>
       </c>
-      <c r="I52" s="11" t="s">
+      <c r="J52" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="J52" s="11" t="s">
+      <c r="K52" s="11" t="s">
         <v>198</v>
-      </c>
-      <c r="K52" s="11" t="s">
-        <v>199</v>
       </c>
       <c r="L52" s="11"/>
       <c r="M52" s="10">
@@ -3854,37 +3854,37 @@
         <v>51</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C53" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="D53" s="10" t="s">
         <v>200</v>
-      </c>
-      <c r="D53" s="10" t="s">
-        <v>201</v>
       </c>
       <c r="E53" s="10">
         <v>6</v>
       </c>
       <c r="F53" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="G53" s="11" t="s">
         <v>207</v>
       </c>
-      <c r="G53" s="11" t="s">
+      <c r="H53" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="H53" s="11" t="s">
-        <v>209</v>
-      </c>
       <c r="I53" s="11" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="J53" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="K53" s="11" t="s">
         <v>205</v>
       </c>
-      <c r="K53" s="11" t="s">
-        <v>206</v>
-      </c>
       <c r="L53" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M53" s="10">
         <v>1</v>
@@ -3896,7 +3896,7 @@
         <v>237</v>
       </c>
       <c r="P53" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="Q53" s="30"/>
     </row>
@@ -3905,31 +3905,31 @@
         <v>52</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C54" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="D54" s="10" t="s">
         <v>210</v>
-      </c>
-      <c r="D54" s="10" t="s">
-        <v>211</v>
       </c>
       <c r="E54" s="10">
         <v>6</v>
       </c>
       <c r="F54" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="G54" s="11" t="s">
         <v>202</v>
       </c>
-      <c r="G54" s="11" t="s">
+      <c r="H54" s="11" t="s">
         <v>203</v>
-      </c>
-      <c r="H54" s="11" t="s">
-        <v>204</v>
       </c>
       <c r="I54" s="11"/>
       <c r="J54" s="11"/>
       <c r="K54" s="11"/>
       <c r="L54" s="11" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="M54" s="10">
         <v>2</v>
@@ -3941,7 +3941,7 @@
         <v>250</v>
       </c>
       <c r="P54" s="11" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="Q54" s="30"/>
     </row>
@@ -3950,37 +3950,37 @@
         <v>53</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C55" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="D55" s="10" t="s">
         <v>213</v>
-      </c>
-      <c r="D55" s="10" t="s">
-        <v>214</v>
       </c>
       <c r="E55" s="10">
         <v>6</v>
       </c>
       <c r="F55" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="G55" s="11" t="s">
         <v>216</v>
       </c>
-      <c r="G55" s="11" t="s">
+      <c r="H55" s="11" t="s">
         <v>217</v>
       </c>
-      <c r="H55" s="11" t="s">
+      <c r="I55" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="J55" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="I55" s="10" t="s">
-        <v>216</v>
-      </c>
-      <c r="J55" s="10" t="s">
+      <c r="K55" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="K55" s="10" t="s">
-        <v>220</v>
-      </c>
       <c r="L55" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="M55" s="10">
         <v>2</v>
@@ -3992,7 +3992,7 @@
         <v>262</v>
       </c>
       <c r="P55" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="Q55" s="30"/>
     </row>
@@ -4001,37 +4001,37 @@
         <v>54</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C56" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="D56" s="10" t="s">
         <v>174</v>
-      </c>
-      <c r="D56" s="10" t="s">
-        <v>175</v>
       </c>
       <c r="E56" s="10">
         <v>6</v>
       </c>
       <c r="F56" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="G56" s="11" t="s">
         <v>176</v>
       </c>
-      <c r="G56" s="11" t="s">
+      <c r="H56" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="I56" s="11" t="s">
         <v>177</v>
       </c>
-      <c r="H56" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="I56" s="11" t="s">
+      <c r="J56" s="11" t="s">
         <v>178</v>
       </c>
-      <c r="J56" s="11" t="s">
-        <v>179</v>
-      </c>
       <c r="K56" s="11" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="L56" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="M56" s="10">
         <v>2</v>
@@ -4043,7 +4043,7 @@
         <v>275</v>
       </c>
       <c r="P56" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Q56" s="30"/>
     </row>
@@ -4052,37 +4052,37 @@
         <v>55</v>
       </c>
       <c r="B57" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="C57" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="C57" s="10" t="s">
+      <c r="D57" s="10" t="s">
         <v>165</v>
-      </c>
-      <c r="D57" s="10" t="s">
-        <v>166</v>
       </c>
       <c r="E57" s="10">
         <v>6</v>
       </c>
       <c r="F57" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="G57" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="G57" s="11" t="s">
+      <c r="H57" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="H57" s="11" t="s">
+      <c r="I57" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="I57" s="11" t="s">
+      <c r="J57" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="J57" s="11" t="s">
+      <c r="K57" s="11" t="s">
         <v>171</v>
       </c>
-      <c r="K57" s="11" t="s">
+      <c r="L57" s="11" t="s">
         <v>172</v>
-      </c>
-      <c r="L57" s="11" t="s">
-        <v>173</v>
       </c>
       <c r="M57" s="10">
         <v>2</v>
@@ -4094,7 +4094,7 @@
         <v>300</v>
       </c>
       <c r="P57" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="Q57" s="30"/>
     </row>

</xml_diff>

<commit_message>
Release 1.2.7: faster views, shop purchases, profile modal, and session sync.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/desafios.xlsx
+++ b/public/resources/desafios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA5DA75D-466E-448D-B835-763C7EC69F36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CB7172E-1E21-4AA1-A157-0768798963E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="312">
   <si>
     <t>nombre</t>
   </si>
@@ -958,6 +958,9 @@
   </si>
   <si>
     <t>Bloodspot</t>
+  </si>
+  <si>
+    <t>The Spectre</t>
   </si>
 </sst>
 </file>
@@ -2561,7 +2564,7 @@
       <c r="J24" s="11"/>
       <c r="K24" s="11"/>
       <c r="L24" s="11" t="s">
-        <v>148</v>
+        <v>311</v>
       </c>
       <c r="M24" s="10">
         <v>1</v>

</xml_diff>